<commit_message>
Improve test for LAST in RAMP in foo
</commit_message>
<xml_diff>
--- a/tests/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
+++ b/tests/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
@@ -1,33 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naqv776\Documents\Research\COPPER\copper_GitHub\issue52_handle_LAST_in_string_fxn\tests\conformance_tests\foo\test_scripts\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56808E0-5EEA-4AA8-8E7E-7B5021D2434D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Script" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Script" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -36,12 +20,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="T5" authorId="0">
       <text>
         <r>
           <rPr>
@@ -49,14 +33,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     "1 total cooling requests remains at time data are recorded since loop output is still &gt;=85%" wording is unclear</t>
         </r>
       </text>
     </comment>
-    <comment ref="U5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="U5" authorId="0">
       <text>
         <r>
           <rPr>
@@ -64,14 +48,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     "0 total cooling requests remains at time data are recorded since loop output is &lt;85%" wording is unclear</t>
         </r>
       </text>
     </comment>
-    <comment ref="AI35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="AI35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -79,14 +63,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;70% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AJ35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="AJ35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -94,14 +78,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;70% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AM35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="AM35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -109,14 +93,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;50% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AW37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AW37" authorId="0">
       <text>
         <r>
           <rPr>
@@ -124,14 +108,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Unlikely that we will be able to get the loop to go to 50% exactly.  This needs to be an inequality</t>
         </r>
       </text>
     </comment>
-    <comment ref="BD37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="BC50" authorId="0">
       <text>
         <r>
           <rPr>
@@ -139,26 +123,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Possibility that the valve jumps above 94% and generates a request in this step
-Reply:
-    As noted, this is a concern that pops up repeatedly and we need to decide how we want to handle is.  See my other comment.
-Reply:
-    decision to leave unchanged for now</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BC50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     This can be simplified to AHUSupAirTempSp+MaxDeltaT since you already assumed heating loop will be 100% based on Vspt
@@ -176,438 +141,474 @@
         </r>
       </text>
     </comment>
+    <comment ref="BD37" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Possibility that the valve jumps above 94% and generates a request in this step
+Reply:
+    As noted, this is a concern that pops up repeatedly and we need to decide how we want to handle is.  See my other comment.
+Reply:
+    decision to leave unchanged for now</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="138">
-  <si>
-    <t>Dummy Test</t>
-  </si>
-  <si>
-    <t>Long Variable Name</t>
-  </si>
-  <si>
-    <t>Variable Name</t>
-  </si>
-  <si>
-    <t>Test Block</t>
-  </si>
-  <si>
-    <t>AA</t>
-  </si>
-  <si>
-    <t>Inputs</t>
-  </si>
-  <si>
-    <t>TestInputs</t>
-  </si>
-  <si>
-    <t>Test Step</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>ts_u1</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>ts_u2</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>ts_u3</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>ts_u4</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>ts_u5</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>ts_u6</t>
-  </si>
-  <si>
-    <t>=ts_u2</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>ts_u7</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>ts_u8</t>
-  </si>
-  <si>
-    <t>=ADD(60;12)</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>ts_u9</t>
-  </si>
-  <si>
-    <t>=MULT(5;13)</t>
-  </si>
-  <si>
-    <t>J</t>
-  </si>
-  <si>
-    <t>ts_u10</t>
-  </si>
-  <si>
-    <t>=SUB(72;4)</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>ts_u11</t>
-  </si>
-  <si>
-    <t>=RAMP(68; 72; 120; 10)</t>
-  </si>
-  <si>
-    <t>=RAMP(68; 72; 60; 10)</t>
-  </si>
-  <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>ts_u12</t>
-  </si>
-  <si>
-    <t>=RAMP(ts_u3; 72; 60; 10)</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>ts_u13</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90)</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>ts_u14</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73)</t>
-  </si>
-  <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>ts_u15</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73; 81)</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>ts_u16</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; ts_u11; 70; 90; 73; 81)</t>
-  </si>
-  <si>
-    <t>Q</t>
-  </si>
-  <si>
-    <t>ts_u17</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>=ADD(ts_u3;12)</t>
-  </si>
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>ts_u18</t>
-  </si>
-  <si>
-    <t>=MULT(ts_u3;12)</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>ts_u19</t>
-  </si>
-  <si>
-    <t>=SUB(ts_u3;12)</t>
-  </si>
-  <si>
-    <t>T</t>
-  </si>
-  <si>
-    <t>ts_u20</t>
-  </si>
-  <si>
-    <t>=PERIODIC(ts_u11; 10)</t>
-  </si>
-  <si>
-    <t>U</t>
-  </si>
-  <si>
-    <t>ts_u21</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u1; 0; ts_u7; ADD(50; 20); 90)</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>ts_u22</t>
-  </si>
-  <si>
-    <t>ON</t>
-  </si>
-  <si>
-    <t>W</t>
-  </si>
-  <si>
-    <t>ts_u23</t>
-  </si>
-  <si>
-    <t>=LAST</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>ts_u24</t>
-  </si>
-  <si>
-    <t>55.04</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>ts_u25</t>
-  </si>
-  <si>
-    <t>Z</t>
-  </si>
-  <si>
-    <t>ts_u26</t>
-  </si>
-  <si>
-    <t>OCCUPIED</t>
-  </si>
-  <si>
-    <t>Conditions for Evaluation of Test Step</t>
-  </si>
-  <si>
-    <t>EvaluationConditions</t>
-  </si>
-  <si>
-    <t>Clock Time</t>
-  </si>
-  <si>
-    <t>ClockTime</t>
-  </si>
-  <si>
-    <t>0:00:30</t>
-  </si>
-  <si>
-    <t>0:01:00</t>
-  </si>
-  <si>
-    <t>VariableName</t>
-  </si>
-  <si>
-    <t>ts_y1</t>
-  </si>
-  <si>
-    <t>ts_y11</t>
-  </si>
-  <si>
-    <t>Variable Value</t>
-  </si>
-  <si>
-    <t>VariableValue</t>
-  </si>
-  <si>
-    <t>&gt;=69</t>
-  </si>
-  <si>
-    <t>&lt;=71</t>
-  </si>
-  <si>
-    <t>&gt;=70</t>
-  </si>
-  <si>
-    <t>Expected Outputs</t>
-  </si>
-  <si>
-    <t>TestOutputs</t>
-  </si>
-  <si>
-    <t>OutputTolerance</t>
-  </si>
-  <si>
-    <t>=ANY</t>
-  </si>
-  <si>
-    <t>ts_y2</t>
-  </si>
-  <si>
-    <t>ts_y3</t>
-  </si>
-  <si>
-    <t>ts_y4</t>
-  </si>
-  <si>
-    <t>ts_y5</t>
-  </si>
-  <si>
-    <t>ts_y6</t>
-  </si>
-  <si>
-    <t>ts_y7</t>
-  </si>
-  <si>
-    <t>ts_y8</t>
-  </si>
-  <si>
-    <t>ts_y9</t>
-  </si>
-  <si>
-    <t>ts_y10</t>
-  </si>
-  <si>
-    <t>ts_y12</t>
-  </si>
-  <si>
-    <t>ts_y13</t>
-  </si>
-  <si>
-    <t>82</t>
-  </si>
-  <si>
-    <t>ts_y14</t>
-  </si>
-  <si>
-    <t>ts_y15</t>
-  </si>
-  <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>ts_y16</t>
-  </si>
-  <si>
-    <t>ts_y17</t>
-  </si>
-  <si>
-    <t>ts_y18</t>
-  </si>
-  <si>
-    <t>ts_y19</t>
-  </si>
-  <si>
-    <t>ts_y20</t>
-  </si>
-  <si>
-    <t>ts_y21</t>
-  </si>
-  <si>
-    <t>ts_y23</t>
-  </si>
-  <si>
-    <t>&gt;50</t>
-  </si>
-  <si>
-    <t>ts_y24</t>
-  </si>
-  <si>
-    <t>&lt;56</t>
-  </si>
-  <si>
-    <t>=RAMP(LAST; 200; 60; 10)</t>
-  </si>
-  <si>
-    <t>200</t>
-  </si>
-  <si>
-    <t>=SUB(LAST;48)</t>
-  </si>
-  <si>
-    <t>=ADD(LAST;55)</t>
-  </si>
-  <si>
-    <t>=MULT(LAST;1)</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 60; LAST; 500; 500; 500)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="137">
+  <si>
+    <t xml:space="preserve">Dummy Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long Variable Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestInputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(LAST;1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ts_u2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 60; LAST; 500; 500; 500)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(LAST; 200; 120; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(60;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(5;13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(LAST;55)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(72;4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(LAST;48)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(68; 72; 120; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(68; 72; 60; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(ts_u3; 72; 60; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73; 81)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; ts_u11; 70; 90; 73; 81)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(ts_u3;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(ts_u3;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(ts_u3;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=PERIODIC(ts_u11; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u1; 0; ts_u7; ADD(50; 20); 90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=LAST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">55.04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OCCUPIED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditions for Evaluation of Test Step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EvaluationConditions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clock Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ClockTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0:00:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0:01:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableValue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;=69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;=71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;=70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected Outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestOutputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OutputTolerance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ANY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;56</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="h:mm:ss"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -617,7 +618,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -675,169 +676,258 @@
     </fill>
   </fills>
   <borders count="3">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
+      <right style="thick"/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thick">
-        <color auto="1"/>
-      </left>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thick"/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+  <cellXfs count="49">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -848,7 +938,6 @@
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -907,78 +996,62 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="DejaVu Sans"/>
-        <a:cs typeface="DejaVu Sans"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="DejaVu Sans"/>
-        <a:cs typeface="DejaVu Sans"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1031,25 +1104,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ61"/>
-  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:CA61"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="64.15625" customWidth="1"/>
-    <col min="2" max="2" width="26.3125" customWidth="1"/>
-    <col min="3" max="3" width="18.47265625" customWidth="1"/>
-    <col min="4" max="6" width="50.68359375" style="1" customWidth="1"/>
-    <col min="7" max="79" width="50.68359375" style="2" customWidth="1"/>
-    <col min="80" max="1024" width="8.83984375" style="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="64.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="50.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="79" min="7" style="2" width="50.68"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="80" style="2" width="8.84"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" s="6" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1149,7 @@
       <c r="BQ1" s="7"/>
       <c r="BR1" s="8"/>
     </row>
-    <row r="2" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1101,7 +1175,7 @@
       <c r="BQ2" s="10"/>
       <c r="BR2" s="11"/>
     </row>
-    <row r="3" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1192,7 +1266,7 @@
       <c r="BZ3" s="4"/>
       <c r="CA3" s="4"/>
     </row>
-    <row r="4" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1289,7 @@
       <c r="BQ4" s="10"/>
       <c r="BR4" s="11"/>
     </row>
-    <row r="5" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1237,7 +1311,7 @@
       <c r="BQ5" s="10"/>
       <c r="BR5" s="11"/>
     </row>
-    <row r="6" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
         <v>1</v>
       </c>
@@ -1342,7 +1416,7 @@
       <c r="BZ6" s="18"/>
       <c r="CA6" s="18"/>
     </row>
-    <row r="7" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
         <v>5</v>
       </c>
@@ -1352,15 +1426,15 @@
       <c r="C7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="24">
-        <f>IF(C6=D6,C7+1,1)</f>
+      <c r="D7" s="24" t="n">
+        <f aca="false">IF(C6=D6,C7+1,1)</f>
         <v>1</v>
       </c>
-      <c r="E7" s="24">
-        <f>IF(D6=E6,D7+1,1)</f>
+      <c r="E7" s="24" t="n">
+        <f aca="false">IF(D6=E6,D7+1,1)</f>
         <v>2</v>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="24" t="n">
         <v>3</v>
       </c>
       <c r="G7" s="24" t="s">
@@ -1449,7 +1523,7 @@
       <c r="BZ7" s="25"/>
       <c r="CA7" s="25"/>
     </row>
-    <row r="8" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
         <v>14</v>
       </c>
@@ -1457,31 +1531,31 @@
         <v>15</v>
       </c>
       <c r="C8" s="32"/>
-      <c r="D8" s="33">
+      <c r="D8" s="33" t="n">
         <v>70</v>
       </c>
-      <c r="E8" s="34">
+      <c r="E8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="F8" s="34">
+      <c r="F8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="H8" s="34">
+      <c r="H8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="L8" s="34">
+      <c r="L8" s="34" t="n">
         <v>70</v>
       </c>
       <c r="M8" s="35"/>
@@ -1552,7 +1626,7 @@
       <c r="BZ8" s="35"/>
       <c r="CA8" s="35"/>
     </row>
-    <row r="9" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
         <v>16</v>
       </c>
@@ -1560,31 +1634,31 @@
         <v>17</v>
       </c>
       <c r="C9" s="32"/>
-      <c r="D9" s="34">
+      <c r="D9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="E9" s="34">
+      <c r="E9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="F9" s="34">
+      <c r="F9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="I9" s="34">
+      <c r="I9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="J9" s="34">
+      <c r="J9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="K9" s="34">
+      <c r="K9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="L9" s="34">
+      <c r="L9" s="34" t="n">
         <v>75</v>
       </c>
       <c r="M9" s="35"/>
@@ -1655,7 +1729,7 @@
       <c r="BZ9" s="35"/>
       <c r="CA9" s="35"/>
     </row>
-    <row r="10" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="s">
         <v>18</v>
       </c>
@@ -1663,31 +1737,31 @@
         <v>19</v>
       </c>
       <c r="C10" s="38"/>
-      <c r="D10" s="34">
+      <c r="D10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="E10" s="34">
+      <c r="E10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="F10" s="34">
+      <c r="F10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="I10" s="34">
+      <c r="I10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="J10" s="34">
+      <c r="J10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="K10" s="34">
+      <c r="K10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="L10" s="34">
+      <c r="L10" s="34" t="n">
         <v>60</v>
       </c>
       <c r="M10" s="35"/>
@@ -1758,7 +1832,7 @@
       <c r="BZ10" s="35"/>
       <c r="CA10" s="35"/>
     </row>
-    <row r="11" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
         <v>20</v>
       </c>
@@ -1766,31 +1840,31 @@
         <v>21</v>
       </c>
       <c r="C11" s="38"/>
-      <c r="D11" s="34">
+      <c r="D11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="E11" s="34">
+      <c r="E11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="F11" s="34">
+      <c r="F11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="H11" s="34">
+      <c r="H11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="I11" s="34">
+      <c r="I11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="J11" s="34">
+      <c r="J11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="K11" s="34">
+      <c r="K11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="L11" s="34">
+      <c r="L11" s="34" t="n">
         <v>90</v>
       </c>
       <c r="M11" s="35"/>
@@ -1861,7 +1935,7 @@
       <c r="BZ11" s="35"/>
       <c r="CA11" s="35"/>
     </row>
-    <row r="12" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
         <v>22</v>
       </c>
@@ -1869,31 +1943,31 @@
         <v>23</v>
       </c>
       <c r="C12" s="32"/>
-      <c r="D12" s="34">
+      <c r="D12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="E12" s="34">
+      <c r="E12" s="34" t="n">
         <v>1000</v>
       </c>
       <c r="F12" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="G12" s="34">
+        <v>24</v>
+      </c>
+      <c r="G12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="I12" s="34">
+      <c r="I12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="J12" s="34">
+      <c r="J12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="K12" s="34">
+      <c r="K12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="L12" s="34">
+      <c r="L12" s="34" t="n">
         <v>1000</v>
       </c>
       <c r="M12" s="35"/>
@@ -1964,39 +2038,39 @@
       <c r="BZ12" s="35"/>
       <c r="CA12" s="35"/>
     </row>
-    <row r="13" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C13" s="38"/>
-      <c r="D13" s="34">
+      <c r="D13" s="34" t="n">
         <v>500</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F13" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="G13" s="34">
+        <v>28</v>
+      </c>
+      <c r="G13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="H13" s="34">
+      <c r="H13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="I13" s="34">
+      <c r="I13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="J13" s="34">
+      <c r="J13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="K13" s="34">
+      <c r="K13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="L13" s="34">
+      <c r="L13" s="34" t="n">
         <v>500</v>
       </c>
       <c r="M13" s="35"/>
@@ -2067,39 +2141,39 @@
       <c r="BZ13" s="35"/>
       <c r="CA13" s="35"/>
     </row>
-    <row r="14" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C14" s="38"/>
-      <c r="D14" s="34">
+      <c r="D14" s="34" t="n">
         <v>100</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="F14" s="34">
+        <v>31</v>
+      </c>
+      <c r="F14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="G14" s="34">
+      <c r="G14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="H14" s="34">
+      <c r="H14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="I14" s="34">
+      <c r="I14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="J14" s="34">
+      <c r="J14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="K14" s="34">
+      <c r="K14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="L14" s="34">
+      <c r="L14" s="34" t="n">
         <v>100</v>
       </c>
       <c r="M14" s="35"/>
@@ -2170,39 +2244,39 @@
       <c r="BZ14" s="35"/>
       <c r="CA14" s="35"/>
     </row>
-    <row r="15" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C15" s="38"/>
-      <c r="D15" s="34">
+      <c r="D15" s="34" t="n">
         <v>200</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="34">
+        <v>34</v>
+      </c>
+      <c r="F15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="I15" s="34">
+      <c r="I15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="J15" s="34">
+      <c r="J15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="K15" s="34">
+      <c r="K15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="L15" s="34">
+      <c r="L15" s="34" t="n">
         <v>200</v>
       </c>
       <c r="M15" s="35"/>
@@ -2273,39 +2347,39 @@
       <c r="BZ15" s="35"/>
       <c r="CA15" s="35"/>
     </row>
-    <row r="16" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C16" s="38"/>
-      <c r="D16" s="34">
+      <c r="D16" s="34" t="n">
         <v>120</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F16" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="G16" s="34">
+        <v>38</v>
+      </c>
+      <c r="G16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="H16" s="34">
+      <c r="H16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="I16" s="34">
+      <c r="I16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="J16" s="34">
+      <c r="J16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="K16" s="34">
+      <c r="K16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="L16" s="34">
+      <c r="L16" s="34" t="n">
         <v>120</v>
       </c>
       <c r="M16" s="35"/>
@@ -2376,39 +2450,39 @@
       <c r="BZ16" s="35"/>
       <c r="CA16" s="35"/>
     </row>
-    <row r="17" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="31" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C17" s="32"/>
-      <c r="D17" s="34">
+      <c r="D17" s="34" t="n">
         <v>20</v>
       </c>
       <c r="E17" s="34" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F17" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="G17" s="34">
+        <v>42</v>
+      </c>
+      <c r="G17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="H17" s="34">
+      <c r="H17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="I17" s="34">
+      <c r="I17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="J17" s="34">
+      <c r="J17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="K17" s="34">
+      <c r="K17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="L17" s="34">
+      <c r="L17" s="34" t="n">
         <v>20</v>
       </c>
       <c r="M17" s="35"/>
@@ -2479,40 +2553,40 @@
       <c r="BZ17" s="35"/>
       <c r="CA17" s="35"/>
     </row>
-    <row r="18" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="31" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C18" s="38"/>
       <c r="D18" s="34" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F18" s="34" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="G18" s="34" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="I18" s="34" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="J18" s="34" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="K18" s="34" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="M18" s="35"/>
       <c r="N18" s="35"/>
@@ -2582,39 +2656,39 @@
       <c r="BZ18" s="35"/>
       <c r="CA18" s="35"/>
     </row>
-    <row r="19" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="31" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C19" s="32"/>
-      <c r="D19" s="34">
+      <c r="D19" s="34" t="n">
         <v>150</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="34">
+        <v>50</v>
+      </c>
+      <c r="F19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="G19" s="34">
+      <c r="G19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="H19" s="34">
+      <c r="H19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="I19" s="34">
+      <c r="I19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="J19" s="34">
+      <c r="J19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="K19" s="34">
+      <c r="K19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="L19" s="34">
+      <c r="L19" s="34" t="n">
         <v>150</v>
       </c>
       <c r="M19" s="35"/>
@@ -2685,39 +2759,39 @@
       <c r="BZ19" s="35"/>
       <c r="CA19" s="35"/>
     </row>
-    <row r="20" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C20" s="32"/>
-      <c r="D20" s="34">
+      <c r="D20" s="34" t="n">
         <v>55</v>
       </c>
       <c r="E20" s="34" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="34">
+        <v>53</v>
+      </c>
+      <c r="F20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G20" s="34">
+      <c r="G20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H20" s="34">
+      <c r="H20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I20" s="34">
+      <c r="I20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J20" s="34">
+      <c r="J20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K20" s="34">
+      <c r="K20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="L20" s="34">
+      <c r="L20" s="34" t="n">
         <v>55</v>
       </c>
       <c r="M20" s="35"/>
@@ -2788,39 +2862,39 @@
       <c r="BZ20" s="35"/>
       <c r="CA20" s="35"/>
     </row>
-    <row r="21" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C21" s="38"/>
-      <c r="D21" s="34">
+      <c r="D21" s="34" t="n">
         <v>72</v>
       </c>
       <c r="E21" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="F21" s="34">
+        <v>56</v>
+      </c>
+      <c r="F21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="G21" s="34">
+      <c r="G21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="H21" s="34">
+      <c r="H21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="I21" s="34">
+      <c r="I21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="J21" s="34">
+      <c r="J21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="K21" s="34">
+      <c r="K21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="L21" s="34">
+      <c r="L21" s="34" t="n">
         <v>72</v>
       </c>
       <c r="M21" s="35"/>
@@ -2891,39 +2965,39 @@
       <c r="BZ21" s="35"/>
       <c r="CA21" s="35"/>
     </row>
-    <row r="22" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="31" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C22" s="38"/>
-      <c r="D22" s="34">
+      <c r="D22" s="34" t="n">
         <v>400</v>
       </c>
       <c r="E22" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="34">
+        <v>59</v>
+      </c>
+      <c r="F22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="G22" s="34">
+      <c r="G22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="H22" s="34">
+      <c r="H22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="I22" s="34">
+      <c r="I22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="J22" s="34">
+      <c r="J22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="K22" s="34">
+      <c r="K22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="L22" s="34">
+      <c r="L22" s="34" t="n">
         <v>400</v>
       </c>
       <c r="M22" s="35"/>
@@ -2994,40 +3068,40 @@
       <c r="BZ22" s="35"/>
       <c r="CA22" s="35"/>
     </row>
-    <row r="23" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="31" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C23" s="32"/>
       <c r="D23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E23" s="34" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="G23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="J23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="K23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="M23" s="35"/>
       <c r="N23" s="35"/>
@@ -3097,40 +3171,40 @@
       <c r="BZ23" s="35"/>
       <c r="CA23" s="35"/>
     </row>
-    <row r="24" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C24" s="32"/>
       <c r="D24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E24" s="34" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="I24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="J24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="K24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="L24" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="M24" s="35"/>
       <c r="N24" s="35"/>
@@ -3200,39 +3274,39 @@
       <c r="BZ24" s="35"/>
       <c r="CA24" s="35"/>
     </row>
-    <row r="25" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="31" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B25" s="31" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C25" s="38"/>
-      <c r="D25" s="34">
+      <c r="D25" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="34" t="s">
-        <v>65</v>
-      </c>
-      <c r="F25" s="34">
+        <v>70</v>
+      </c>
+      <c r="F25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="34">
+      <c r="G25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H25" s="34">
+      <c r="H25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I25" s="34">
+      <c r="I25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J25" s="34">
+      <c r="J25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K25" s="34">
+      <c r="K25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L25" s="34">
+      <c r="L25" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M25" s="35"/>
@@ -3303,39 +3377,39 @@
       <c r="BZ25" s="35"/>
       <c r="CA25" s="35"/>
     </row>
-    <row r="26" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="31" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B26" s="31" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C26" s="38"/>
-      <c r="D26" s="34">
+      <c r="D26" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="F26" s="34">
+        <v>73</v>
+      </c>
+      <c r="F26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="34">
+      <c r="G26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="34">
+      <c r="H26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I26" s="34">
+      <c r="I26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J26" s="34">
+      <c r="J26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K26" s="34">
+      <c r="K26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L26" s="34">
+      <c r="L26" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M26" s="35"/>
@@ -3406,39 +3480,39 @@
       <c r="BZ26" s="35"/>
       <c r="CA26" s="35"/>
     </row>
-    <row r="27" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="31" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B27" s="31" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C27" s="32"/>
-      <c r="D27" s="34">
+      <c r="D27" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="F27" s="34">
+        <v>76</v>
+      </c>
+      <c r="F27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="34">
+      <c r="G27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="34">
+      <c r="H27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I27" s="34">
+      <c r="I27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="34">
+      <c r="J27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K27" s="34">
+      <c r="K27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L27" s="34">
+      <c r="L27" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M27" s="35"/>
@@ -3509,39 +3583,39 @@
       <c r="BZ27" s="35"/>
       <c r="CA27" s="35"/>
     </row>
-    <row r="28" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="31" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B28" s="31" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C28" s="32"/>
-      <c r="D28" s="34">
+      <c r="D28" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="34" t="s">
-        <v>74</v>
-      </c>
-      <c r="F28" s="34">
+        <v>79</v>
+      </c>
+      <c r="F28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="34">
+      <c r="G28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="34">
+      <c r="H28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I28" s="34">
+      <c r="I28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J28" s="34">
+      <c r="J28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K28" s="34">
+      <c r="K28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L28" s="34">
+      <c r="L28" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M28" s="35"/>
@@ -3612,40 +3686,40 @@
       <c r="BZ28" s="35"/>
       <c r="CA28" s="35"/>
     </row>
-    <row r="29" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B29" s="31" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C29" s="38"/>
       <c r="D29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="I29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="J29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="K29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L29" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="M29" s="35"/>
       <c r="N29" s="35"/>
@@ -3715,40 +3789,40 @@
       <c r="BZ29" s="35"/>
       <c r="CA29" s="35"/>
     </row>
-    <row r="30" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="31" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B30" s="31" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C30" s="38"/>
-      <c r="D30" s="34">
+      <c r="D30" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="E30" s="34">
+      <c r="E30" s="34" t="n">
         <v>55</v>
       </c>
       <c r="F30" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="G30" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="I30" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="J30" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="K30" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L30" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="M30" s="35"/>
       <c r="N30" s="35"/>
@@ -3818,40 +3892,40 @@
       <c r="BZ30" s="35"/>
       <c r="CA30" s="35"/>
     </row>
-    <row r="31" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="31" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B31" s="31" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C31" s="38"/>
-      <c r="D31" s="34">
+      <c r="D31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="F31" s="34">
+      <c r="F31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G31" s="34">
+      <c r="G31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H31" s="34">
+      <c r="H31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I31" s="34">
+      <c r="I31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J31" s="34">
+      <c r="J31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K31" s="34">
+      <c r="K31" s="34" t="n">
         <v>55</v>
       </c>
       <c r="L31" s="34" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="M31" s="35"/>
       <c r="N31" s="35"/>
@@ -3921,40 +3995,40 @@
       <c r="BZ31" s="35"/>
       <c r="CA31" s="35"/>
     </row>
-    <row r="32" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B32" s="31" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C32" s="32"/>
       <c r="D32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="I32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="J32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="K32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L32" s="34" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="M32" s="35"/>
       <c r="N32" s="35"/>
@@ -4024,40 +4098,40 @@
       <c r="BZ32" s="35"/>
       <c r="CA32" s="35"/>
     </row>
-    <row r="33" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="31" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B33" s="31" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C33" s="38"/>
       <c r="D33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="I33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="J33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="K33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="L33" s="34" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="M33" s="35"/>
       <c r="N33" s="35"/>
@@ -4127,12 +4201,12 @@
       <c r="BZ33" s="35"/>
       <c r="CA33" s="35"/>
     </row>
-    <row r="34" spans="1:79" s="41" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" s="41" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="39" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B34" s="39" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C34" s="15"/>
       <c r="D34" s="40"/>
@@ -4153,40 +4227,40 @@
       <c r="BQ34" s="42"/>
       <c r="BR34" s="43"/>
     </row>
-    <row r="35" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="31" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B35" s="31" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C35" s="32"/>
       <c r="D35" s="33" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F35" s="33" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="G35" s="33" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="H35" s="33" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="I35" s="33" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="J35" s="33" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="K35" s="33" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="L35" s="33" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="M35" s="44"/>
       <c r="N35" s="44"/>
@@ -4256,31 +4330,31 @@
       <c r="BZ35" s="44"/>
       <c r="CA35" s="44"/>
     </row>
-    <row r="36" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="47" t="s">
         <v>2</v>
       </c>
       <c r="B36" s="47" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C36" s="38"/>
       <c r="D36" s="33"/>
       <c r="E36" s="33"/>
       <c r="F36" s="33"/>
       <c r="G36" s="33" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H36" s="33" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I36" s="33" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J36" s="33" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="K36" s="33" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="L36" s="33"/>
       <c r="M36" s="35"/>
@@ -4351,31 +4425,31 @@
       <c r="BZ36" s="35"/>
       <c r="CA36" s="35"/>
     </row>
-    <row r="37" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="47" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B37" s="47" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C37" s="38"/>
       <c r="D37" s="33"/>
       <c r="E37" s="33"/>
       <c r="F37" s="33"/>
       <c r="G37" s="33" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="H37" s="33" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I37" s="33" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="J37" s="33" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="K37" s="33" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="L37" s="33"/>
       <c r="M37" s="35"/>
@@ -4446,15 +4520,15 @@
       <c r="BZ37" s="35"/>
       <c r="CA37" s="35"/>
     </row>
-    <row r="38" spans="1:79" s="41" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" s="41" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="39" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
@@ -4474,41 +4548,41 @@
       <c r="BQ38" s="42"/>
       <c r="BR38" s="43"/>
     </row>
-    <row r="39" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="31" t="s">
         <v>14</v>
       </c>
       <c r="B39" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="C39" s="38">
+        <v>101</v>
+      </c>
+      <c r="C39" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E39" s="33">
+        <v>111</v>
+      </c>
+      <c r="E39" s="33" t="n">
         <v>70</v>
       </c>
-      <c r="F39" s="34">
+      <c r="F39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="G39" s="34">
+      <c r="G39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="H39" s="34">
+      <c r="H39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="I39" s="34">
+      <c r="I39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="J39" s="34">
+      <c r="J39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="K39" s="34">
+      <c r="K39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="L39" s="34">
+      <c r="L39" s="34" t="n">
         <v>70</v>
       </c>
       <c r="M39" s="35"/>
@@ -4579,41 +4653,41 @@
       <c r="BZ39" s="35"/>
       <c r="CA39" s="35"/>
     </row>
-    <row r="40" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="31" t="s">
         <v>16</v>
       </c>
       <c r="B40" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="C40" s="38">
+        <v>112</v>
+      </c>
+      <c r="C40" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E40" s="33">
+        <v>111</v>
+      </c>
+      <c r="E40" s="33" t="n">
         <v>75</v>
       </c>
-      <c r="F40" s="34">
+      <c r="F40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="G40" s="34">
+      <c r="G40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="H40" s="34">
+      <c r="H40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="I40" s="34">
+      <c r="I40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="J40" s="34">
+      <c r="J40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="K40" s="34">
+      <c r="K40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="L40" s="34">
+      <c r="L40" s="34" t="n">
         <v>75</v>
       </c>
       <c r="M40" s="35"/>
@@ -4684,41 +4758,41 @@
       <c r="BZ40" s="35"/>
       <c r="CA40" s="35"/>
     </row>
-    <row r="41" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="31" t="s">
         <v>18</v>
       </c>
       <c r="B41" s="31" t="s">
-        <v>108</v>
-      </c>
-      <c r="C41" s="38">
+        <v>113</v>
+      </c>
+      <c r="C41" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E41" s="33">
+        <v>111</v>
+      </c>
+      <c r="E41" s="33" t="n">
         <v>60</v>
       </c>
-      <c r="F41" s="34">
+      <c r="F41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="G41" s="34">
+      <c r="G41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="H41" s="34">
+      <c r="H41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="I41" s="34">
+      <c r="I41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="J41" s="34">
+      <c r="J41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="K41" s="34">
+      <c r="K41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="L41" s="34">
+      <c r="L41" s="34" t="n">
         <v>60</v>
       </c>
       <c r="M41" s="35"/>
@@ -4789,41 +4863,41 @@
       <c r="BZ41" s="35"/>
       <c r="CA41" s="35"/>
     </row>
-    <row r="42" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="31" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="31" t="s">
-        <v>109</v>
-      </c>
-      <c r="C42" s="38">
+        <v>114</v>
+      </c>
+      <c r="C42" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E42" s="33">
+        <v>111</v>
+      </c>
+      <c r="E42" s="33" t="n">
         <v>90</v>
       </c>
-      <c r="F42" s="34">
+      <c r="F42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="G42" s="34">
+      <c r="G42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="H42" s="34">
+      <c r="H42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="I42" s="34">
+      <c r="I42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="J42" s="34">
+      <c r="J42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="K42" s="34">
+      <c r="K42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="L42" s="34">
+      <c r="L42" s="34" t="n">
         <v>90</v>
       </c>
       <c r="M42" s="35"/>
@@ -4894,41 +4968,41 @@
       <c r="BZ42" s="35"/>
       <c r="CA42" s="35"/>
     </row>
-    <row r="43" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="31" t="s">
         <v>22</v>
       </c>
       <c r="B43" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="C43" s="38">
+        <v>115</v>
+      </c>
+      <c r="C43" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E43" s="33">
+        <v>111</v>
+      </c>
+      <c r="E43" s="33" t="n">
         <v>1000</v>
       </c>
-      <c r="F43" s="34">
+      <c r="F43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="G43" s="34">
+      <c r="G43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="H43" s="34">
+      <c r="H43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="I43" s="34">
+      <c r="I43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="J43" s="34">
+      <c r="J43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="K43" s="34">
+      <c r="K43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="L43" s="34">
+      <c r="L43" s="34" t="n">
         <v>1000</v>
       </c>
       <c r="M43" s="35"/>
@@ -4999,41 +5073,41 @@
       <c r="BZ43" s="35"/>
       <c r="CA43" s="35"/>
     </row>
-    <row r="44" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="31" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B44" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="C44" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="38">
-        <v>0</v>
-      </c>
-      <c r="D44" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E44" s="33">
+      <c r="E44" s="33" t="n">
         <v>75</v>
       </c>
-      <c r="F44" s="34">
+      <c r="F44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="G44" s="34">
+      <c r="G44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="H44" s="34">
+      <c r="H44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="I44" s="34">
+      <c r="I44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="J44" s="34">
+      <c r="J44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="K44" s="34">
+      <c r="K44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="L44" s="34">
+      <c r="L44" s="34" t="n">
         <v>500</v>
       </c>
       <c r="M44" s="35"/>
@@ -5104,41 +5178,41 @@
       <c r="BZ44" s="35"/>
       <c r="CA44" s="35"/>
     </row>
-    <row r="45" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="31" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B45" s="31" t="s">
-        <v>112</v>
-      </c>
-      <c r="C45" s="38">
+        <v>117</v>
+      </c>
+      <c r="C45" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E45" s="33" t="s">
-        <v>133</v>
-      </c>
-      <c r="F45" s="34">
+        <v>111</v>
+      </c>
+      <c r="E45" s="48" t="n">
+        <v>150</v>
+      </c>
+      <c r="F45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="G45" s="34">
+      <c r="G45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="H45" s="34">
+      <c r="H45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="I45" s="34">
+      <c r="I45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="J45" s="34">
+      <c r="J45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="K45" s="34">
+      <c r="K45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="L45" s="34">
+      <c r="L45" s="34" t="n">
         <v>100</v>
       </c>
       <c r="M45" s="35"/>
@@ -5209,41 +5283,41 @@
       <c r="BZ45" s="35"/>
       <c r="CA45" s="35"/>
     </row>
-    <row r="46" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="31" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B46" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="C46" s="38">
+        <v>118</v>
+      </c>
+      <c r="C46" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E46" s="33">
+        <v>111</v>
+      </c>
+      <c r="E46" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F46" s="34">
+      <c r="F46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="G46" s="34">
+      <c r="G46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="H46" s="34">
+      <c r="H46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="I46" s="34">
+      <c r="I46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="J46" s="34">
+      <c r="J46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="K46" s="34">
+      <c r="K46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="L46" s="34">
+      <c r="L46" s="34" t="n">
         <v>200</v>
       </c>
       <c r="M46" s="35"/>
@@ -5314,41 +5388,41 @@
       <c r="BZ46" s="35"/>
       <c r="CA46" s="35"/>
     </row>
-    <row r="47" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="31" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B47" s="31" t="s">
-        <v>114</v>
-      </c>
-      <c r="C47" s="38">
+        <v>119</v>
+      </c>
+      <c r="C47" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E47" s="33">
+        <v>111</v>
+      </c>
+      <c r="E47" s="33" t="n">
         <v>65</v>
       </c>
-      <c r="F47" s="34">
+      <c r="F47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="G47" s="34">
+      <c r="G47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="H47" s="34">
+      <c r="H47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="I47" s="34">
+      <c r="I47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="J47" s="34">
+      <c r="J47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="K47" s="34">
+      <c r="K47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="L47" s="34">
+      <c r="L47" s="34" t="n">
         <v>120</v>
       </c>
       <c r="M47" s="35"/>
@@ -5419,41 +5493,41 @@
       <c r="BZ47" s="35"/>
       <c r="CA47" s="35"/>
     </row>
-    <row r="48" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="31" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B48" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="C48" s="38">
+        <v>120</v>
+      </c>
+      <c r="C48" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E48" s="33">
+        <v>111</v>
+      </c>
+      <c r="E48" s="33" t="n">
         <v>68</v>
       </c>
-      <c r="F48" s="34">
+      <c r="F48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="G48" s="34">
+      <c r="G48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="H48" s="34">
+      <c r="H48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="I48" s="34">
+      <c r="I48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="J48" s="34">
+      <c r="J48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="K48" s="34">
+      <c r="K48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="L48" s="34">
+      <c r="L48" s="34" t="n">
         <v>20</v>
       </c>
       <c r="M48" s="35"/>
@@ -5524,41 +5598,41 @@
       <c r="BZ48" s="35"/>
       <c r="CA48" s="35"/>
     </row>
-    <row r="49" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="31" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B49" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="C49" s="38">
+        <v>102</v>
+      </c>
+      <c r="C49" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E49" s="33">
+        <v>111</v>
+      </c>
+      <c r="E49" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F49" s="34">
+      <c r="F49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="G49" s="34">
+      <c r="G49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="H49" s="34">
+      <c r="H49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="I49" s="34">
+      <c r="I49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="J49" s="34">
+      <c r="J49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="K49" s="34">
+      <c r="K49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="L49" s="34">
+      <c r="L49" s="34" t="n">
         <v>70</v>
       </c>
       <c r="M49" s="35"/>
@@ -5629,41 +5703,41 @@
       <c r="BZ49" s="35"/>
       <c r="CA49" s="35"/>
     </row>
-    <row r="50" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="31" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B50" s="31" t="s">
-        <v>116</v>
-      </c>
-      <c r="C50" s="38">
+        <v>121</v>
+      </c>
+      <c r="C50" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E50" s="33">
+        <v>111</v>
+      </c>
+      <c r="E50" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F50" s="34">
+      <c r="F50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="G50" s="34">
+      <c r="G50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="H50" s="34">
+      <c r="H50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="I50" s="34">
+      <c r="I50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="J50" s="34">
+      <c r="J50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="K50" s="34">
+      <c r="K50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="L50" s="34">
+      <c r="L50" s="34" t="n">
         <v>150</v>
       </c>
       <c r="M50" s="35"/>
@@ -5734,41 +5808,41 @@
       <c r="BZ50" s="35"/>
       <c r="CA50" s="35"/>
     </row>
-    <row r="51" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="31" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B51" s="31" t="s">
-        <v>117</v>
-      </c>
-      <c r="C51" s="38">
+        <v>122</v>
+      </c>
+      <c r="C51" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="33" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E51" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="F51" s="34">
+        <v>123</v>
+      </c>
+      <c r="F51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G51" s="34">
+      <c r="G51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H51" s="34">
+      <c r="H51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I51" s="34">
+      <c r="I51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J51" s="34">
+      <c r="J51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K51" s="34">
+      <c r="K51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="L51" s="34">
+      <c r="L51" s="34" t="n">
         <v>55</v>
       </c>
       <c r="M51" s="35"/>
@@ -5839,41 +5913,41 @@
       <c r="BZ51" s="35"/>
       <c r="CA51" s="35"/>
     </row>
-    <row r="52" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="31" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B52" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="C52" s="38">
+        <v>124</v>
+      </c>
+      <c r="C52" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="33" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E52" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="F52" s="34">
+        <v>123</v>
+      </c>
+      <c r="F52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="G52" s="34">
+      <c r="G52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="H52" s="34">
+      <c r="H52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="I52" s="34">
+      <c r="I52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="J52" s="34">
+      <c r="J52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="K52" s="34">
+      <c r="K52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="L52" s="34">
+      <c r="L52" s="34" t="n">
         <v>72</v>
       </c>
       <c r="M52" s="35"/>
@@ -5944,41 +6018,41 @@
       <c r="BZ52" s="35"/>
       <c r="CA52" s="35"/>
     </row>
-    <row r="53" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="31" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B53" s="31" t="s">
-        <v>120</v>
-      </c>
-      <c r="C53" s="38">
+        <v>125</v>
+      </c>
+      <c r="C53" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="33" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E53" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="F53" s="34">
+        <v>126</v>
+      </c>
+      <c r="F53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="G53" s="34">
+      <c r="G53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="H53" s="34">
+      <c r="H53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="I53" s="34">
+      <c r="I53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="J53" s="34">
+      <c r="J53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="K53" s="34">
+      <c r="K53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="L53" s="34">
+      <c r="L53" s="34" t="n">
         <v>400</v>
       </c>
       <c r="M53" s="35"/>
@@ -6049,42 +6123,42 @@
       <c r="BZ53" s="35"/>
       <c r="CA53" s="35"/>
     </row>
-    <row r="54" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="31" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B54" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="C54" s="38">
+        <v>127</v>
+      </c>
+      <c r="C54" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="33" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E54" s="33" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F54" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="G54" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H54" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="I54" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="J54" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="K54" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="L54" s="34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="M54" s="35"/>
       <c r="N54" s="35"/>
@@ -6154,42 +6228,42 @@
       <c r="BZ54" s="35"/>
       <c r="CA54" s="35"/>
     </row>
-    <row r="55" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="31" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B55" s="31" t="s">
-        <v>123</v>
-      </c>
-      <c r="C55" s="38">
+        <v>128</v>
+      </c>
+      <c r="C55" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E55" s="33">
+        <v>111</v>
+      </c>
+      <c r="E55" s="33" t="n">
         <v>72</v>
       </c>
       <c r="F55" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G55" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="H55" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="I55" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="J55" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="K55" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="L55" s="34" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="M55" s="35"/>
       <c r="N55" s="35"/>
@@ -6259,41 +6333,41 @@
       <c r="BZ55" s="35"/>
       <c r="CA55" s="35"/>
     </row>
-    <row r="56" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="31" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B56" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="C56" s="38">
+        <v>129</v>
+      </c>
+      <c r="C56" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E56" s="33">
+        <v>111</v>
+      </c>
+      <c r="E56" s="33" t="n">
         <v>720</v>
       </c>
-      <c r="F56" s="34">
+      <c r="F56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G56" s="34">
+      <c r="G56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H56" s="34">
+      <c r="H56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I56" s="34">
+      <c r="I56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J56" s="34">
+      <c r="J56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K56" s="34">
+      <c r="K56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L56" s="34">
+      <c r="L56" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M56" s="35"/>
@@ -6364,41 +6438,41 @@
       <c r="BZ56" s="35"/>
       <c r="CA56" s="35"/>
     </row>
-    <row r="57" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="31" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B57" s="31" t="s">
-        <v>125</v>
-      </c>
-      <c r="C57" s="32">
+        <v>130</v>
+      </c>
+      <c r="C57" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E57" s="33">
+        <v>111</v>
+      </c>
+      <c r="E57" s="33" t="n">
         <v>48</v>
       </c>
-      <c r="F57" s="34">
+      <c r="F57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G57" s="34">
+      <c r="G57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H57" s="34">
+      <c r="H57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I57" s="34">
+      <c r="I57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J57" s="34">
+      <c r="J57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K57" s="34">
+      <c r="K57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L57" s="34">
+      <c r="L57" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M57" s="35"/>
@@ -6469,41 +6543,41 @@
       <c r="BZ57" s="35"/>
       <c r="CA57" s="35"/>
     </row>
-    <row r="58" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="31" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B58" s="31" t="s">
-        <v>126</v>
-      </c>
-      <c r="C58" s="32">
+        <v>131</v>
+      </c>
+      <c r="C58" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E58" s="33">
+        <v>111</v>
+      </c>
+      <c r="E58" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F58" s="34">
+      <c r="F58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="34">
+      <c r="G58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H58" s="34">
+      <c r="H58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I58" s="34">
+      <c r="I58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J58" s="34">
+      <c r="J58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K58" s="34">
+      <c r="K58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L58" s="34">
+      <c r="L58" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M58" s="35"/>
@@ -6574,41 +6648,41 @@
       <c r="BZ58" s="35"/>
       <c r="CA58" s="35"/>
     </row>
-    <row r="59" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="31" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B59" s="31" t="s">
-        <v>127</v>
-      </c>
-      <c r="C59" s="38">
+        <v>132</v>
+      </c>
+      <c r="C59" s="38" t="n">
         <v>0</v>
       </c>
       <c r="D59" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="E59" s="33">
+        <v>111</v>
+      </c>
+      <c r="E59" s="33" t="n">
         <v>84</v>
       </c>
-      <c r="F59" s="34">
+      <c r="F59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G59" s="34">
+      <c r="G59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H59" s="34">
+      <c r="H59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I59" s="34">
+      <c r="I59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J59" s="34">
+      <c r="J59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K59" s="34">
+      <c r="K59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L59" s="34">
+      <c r="L59" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M59" s="35"/>
@@ -6679,41 +6753,41 @@
       <c r="BZ59" s="35"/>
       <c r="CA59" s="35"/>
     </row>
-    <row r="60" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="31" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B60" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="C60" s="32">
+        <v>133</v>
+      </c>
+      <c r="C60" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D60" s="33" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E60" s="33" t="s">
-        <v>129</v>
-      </c>
-      <c r="F60" s="34">
+        <v>134</v>
+      </c>
+      <c r="F60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G60" s="34">
+      <c r="G60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H60" s="34">
+      <c r="H60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I60" s="34">
+      <c r="I60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J60" s="34">
+      <c r="J60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K60" s="34">
+      <c r="K60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="L60" s="34">
+      <c r="L60" s="34" t="n">
         <v>55</v>
       </c>
       <c r="M60" s="35"/>
@@ -6784,42 +6858,42 @@
       <c r="BZ60" s="35"/>
       <c r="CA60" s="35"/>
     </row>
-    <row r="61" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="31" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B61" s="31" t="s">
-        <v>130</v>
-      </c>
-      <c r="C61" s="32">
+        <v>135</v>
+      </c>
+      <c r="C61" s="32" t="n">
         <v>0.05</v>
       </c>
       <c r="D61" s="33" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E61" s="33" t="s">
-        <v>131</v>
-      </c>
-      <c r="F61" s="34">
+        <v>136</v>
+      </c>
+      <c r="F61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G61" s="34">
+      <c r="G61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H61" s="34">
+      <c r="H61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I61" s="34">
+      <c r="I61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J61" s="34">
+      <c r="J61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K61" s="34">
+      <c r="K61" s="34" t="n">
         <v>55</v>
       </c>
       <c r="L61" s="34" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="M61" s="35"/>
       <c r="N61" s="35"/>
@@ -6891,12 +6965,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="M8:ZZ33 M39:ZZ61">
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>#REF!&lt;&gt;M8</formula>
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>#ref!&lt;&gt;M8</formula>
     </cfRule>
   </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Test.py and TestScript-foo.xlsx
</commit_message>
<xml_diff>
--- a/tests/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
+++ b/tests/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
@@ -1,17 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naqv776\Documents\Research\COPPER\copper_GitHub\issue52_handle_LAST_in_string_fxn\tests\conformance_tests\foo\test_scripts\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EEC7718-6583-435C-9F28-898E41FB990C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Script" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Test Script" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -20,12 +36,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="T5" authorId="0">
+    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -33,14 +49,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Threaded comment]
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     "1 total cooling requests remains at time data are recorded since loop output is still &gt;=85%" wording is unclear</t>
         </r>
       </text>
     </comment>
-    <comment ref="U5" authorId="0">
+    <comment ref="U5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -48,14 +64,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Threaded comment]
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     "0 total cooling requests remains at time data are recorded since loop output is &lt;85%" wording is unclear</t>
         </r>
       </text>
     </comment>
-    <comment ref="AI35" authorId="0">
+    <comment ref="AI35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -63,14 +79,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Threaded comment]
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;70% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AJ35" authorId="0">
+    <comment ref="AJ35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -78,14 +94,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Threaded comment]
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;70% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AM35" authorId="0">
+    <comment ref="AM35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -93,14 +109,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Threaded comment]
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;50% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AW37" authorId="0">
+    <comment ref="AW37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -108,14 +124,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Threaded comment]
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Unlikely that we will be able to get the loop to go to 50% exactly.  This needs to be an inequality</t>
         </r>
       </text>
     </comment>
-    <comment ref="BC50" authorId="0">
+    <comment ref="BD37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -123,7 +139,26 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Threaded comment]
+          <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Possibility that the valve jumps above 94% and generates a request in this step
+Reply:
+    As noted, this is a concern that pops up repeatedly and we need to decide how we want to handle is.  See my other comment.
+Reply:
+    decision to leave unchanged for now</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="BC50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     This can be simplified to AHUSupAirTempSp+MaxDeltaT since you already assumed heating loop will be 100% based on Vspt
@@ -141,474 +176,438 @@
         </r>
       </text>
     </comment>
-    <comment ref="BD37" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Possibility that the valve jumps above 94% and generates a request in this step
-Reply:
-    As noted, this is a concern that pops up repeatedly and we need to decide how we want to handle is.  See my other comment.
-Reply:
-    decision to leave unchanged for now</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="137">
-  <si>
-    <t xml:space="preserve">Dummy Test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long Variable Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variable Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test Block</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TestInputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test Step</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=MULT(LAST;1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=ts_u2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 60; LAST; 500; 500; 500)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=RAMP(LAST; 200; 120; 10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=ADD(60;12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=MULT(5;13)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=ADD(LAST;55)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=SUB(72;4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=SUB(LAST;48)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=RAMP(68; 72; 120; 10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=RAMP(68; 72; 60; 10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=RAMP(ts_u3; 72; 60; 10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73; 81)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; ts_u11; 70; 90; 73; 81)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=ADD(ts_u3;12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=MULT(ts_u3;12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=SUB(ts_u3;12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=PERIODIC(ts_u11; 10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=INTERPOLATE(ts_u1; 0; ts_u7; ADD(50; 20); 90)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ON</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=LAST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">55.04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_u26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCCUPIED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conditions for Evaluation of Test Step</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EvaluationConditions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clock Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ClockTime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0:00:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0:01:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VariableName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variable Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VariableValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt;=69</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;=71</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt;=70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expected Outputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TestOutputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OutputTolerance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">=ANY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">82</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">81</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt;50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ts_y24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;56</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="138">
+  <si>
+    <t>Dummy Test</t>
+  </si>
+  <si>
+    <t>Long Variable Name</t>
+  </si>
+  <si>
+    <t>Variable Name</t>
+  </si>
+  <si>
+    <t>Test Block</t>
+  </si>
+  <si>
+    <t>AA</t>
+  </si>
+  <si>
+    <t>Inputs</t>
+  </si>
+  <si>
+    <t>TestInputs</t>
+  </si>
+  <si>
+    <t>Test Step</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>ts_u1</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>ts_u2</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>ts_u3</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>ts_u4</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>ts_u5</t>
+  </si>
+  <si>
+    <t>=MULT(LAST;1)</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>ts_u6</t>
+  </si>
+  <si>
+    <t>=ts_u2</t>
+  </si>
+  <si>
+    <t>=INTERPOLATE(ts_u3; 0; 60; LAST; 500; 500; 500)</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>ts_u7</t>
+  </si>
+  <si>
+    <t>=RAMP(LAST; 200; 120; 10)</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>ts_u8</t>
+  </si>
+  <si>
+    <t>=ADD(60;12)</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>ts_u9</t>
+  </si>
+  <si>
+    <t>=MULT(5;13)</t>
+  </si>
+  <si>
+    <t>=ADD(LAST;55)</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>ts_u10</t>
+  </si>
+  <si>
+    <t>=SUB(72;4)</t>
+  </si>
+  <si>
+    <t>=SUB(LAST;48)</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>ts_u11</t>
+  </si>
+  <si>
+    <t>=RAMP(68; 72; 120; 10)</t>
+  </si>
+  <si>
+    <t>=RAMP(68; 72; 60; 10)</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>ts_u12</t>
+  </si>
+  <si>
+    <t>=RAMP(ts_u3; 72; 60; 10)</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>ts_u13</t>
+  </si>
+  <si>
+    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90)</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>ts_u14</t>
+  </si>
+  <si>
+    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73)</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>ts_u15</t>
+  </si>
+  <si>
+    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73; 81)</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>ts_u16</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>=INTERPOLATE(ts_u3; 0; ts_u11; 70; 90; 73; 81)</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>ts_u17</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>=ADD(ts_u3;12)</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>ts_u18</t>
+  </si>
+  <si>
+    <t>=MULT(ts_u3;12)</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>ts_u19</t>
+  </si>
+  <si>
+    <t>=SUB(ts_u3;12)</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>ts_u20</t>
+  </si>
+  <si>
+    <t>=PERIODIC(ts_u11; 10)</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>ts_u21</t>
+  </si>
+  <si>
+    <t>=INTERPOLATE(ts_u1; 0; ts_u7; ADD(50; 20); 90)</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>ts_u22</t>
+  </si>
+  <si>
+    <t>ON</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>ts_u23</t>
+  </si>
+  <si>
+    <t>=LAST</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>ts_u24</t>
+  </si>
+  <si>
+    <t>55.04</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>ts_u25</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>ts_u26</t>
+  </si>
+  <si>
+    <t>OCCUPIED</t>
+  </si>
+  <si>
+    <t>Conditions for Evaluation of Test Step</t>
+  </si>
+  <si>
+    <t>EvaluationConditions</t>
+  </si>
+  <si>
+    <t>Clock Time</t>
+  </si>
+  <si>
+    <t>ClockTime</t>
+  </si>
+  <si>
+    <t>0:00:30</t>
+  </si>
+  <si>
+    <t>0:01:00</t>
+  </si>
+  <si>
+    <t>VariableName</t>
+  </si>
+  <si>
+    <t>ts_y1</t>
+  </si>
+  <si>
+    <t>ts_y11</t>
+  </si>
+  <si>
+    <t>Variable Value</t>
+  </si>
+  <si>
+    <t>VariableValue</t>
+  </si>
+  <si>
+    <t>&gt;=69</t>
+  </si>
+  <si>
+    <t>&lt;=71</t>
+  </si>
+  <si>
+    <t>&gt;=70</t>
+  </si>
+  <si>
+    <t>Expected Outputs</t>
+  </si>
+  <si>
+    <t>TestOutputs</t>
+  </si>
+  <si>
+    <t>OutputTolerance</t>
+  </si>
+  <si>
+    <t>=ANY</t>
+  </si>
+  <si>
+    <t>ts_y2</t>
+  </si>
+  <si>
+    <t>ts_y3</t>
+  </si>
+  <si>
+    <t>ts_y4</t>
+  </si>
+  <si>
+    <t>ts_y5</t>
+  </si>
+  <si>
+    <t>ts_y6</t>
+  </si>
+  <si>
+    <t>ts_y7</t>
+  </si>
+  <si>
+    <t>ts_y8</t>
+  </si>
+  <si>
+    <t>ts_y9</t>
+  </si>
+  <si>
+    <t>ts_y10</t>
+  </si>
+  <si>
+    <t>ts_y12</t>
+  </si>
+  <si>
+    <t>ts_y13</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>ts_y14</t>
+  </si>
+  <si>
+    <t>ts_y15</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>ts_y16</t>
+  </si>
+  <si>
+    <t>ts_y17</t>
+  </si>
+  <si>
+    <t>ts_y18</t>
+  </si>
+  <si>
+    <t>ts_y19</t>
+  </si>
+  <si>
+    <t>ts_y20</t>
+  </si>
+  <si>
+    <t>ts_y21</t>
+  </si>
+  <si>
+    <t>ts_y23</t>
+  </si>
+  <si>
+    <t>&gt;50</t>
+  </si>
+  <si>
+    <t>ts_y24</t>
+  </si>
+  <si>
+    <t>&lt;56</t>
+  </si>
+  <si>
+    <t>=INTERPOLATE(LAST; 0; 162; 0; 800)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
-    <numFmt numFmtId="166" formatCode="h:mm:ss"/>
-  </numFmts>
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -618,7 +617,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -676,258 +675,169 @@
     </fill>
   </fills>
   <borders count="3">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
-      <right style="thick"/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thick"/>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="48">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="49">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -938,6 +848,7 @@
       </fill>
     </dxf>
   </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -996,62 +907,78 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1104,26 +1031,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:CA61"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AMJ61"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="64.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="50.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="79" min="7" style="2" width="50.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="80" style="2" width="8.84"/>
+    <col min="1" max="1" width="64.15625" customWidth="1"/>
+    <col min="2" max="2" width="26.3125" customWidth="1"/>
+    <col min="3" max="3" width="18.47265625" customWidth="1"/>
+    <col min="4" max="6" width="50.68359375" style="1" customWidth="1"/>
+    <col min="7" max="79" width="50.68359375" style="2" customWidth="1"/>
+    <col min="80" max="1024" width="8.83984375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:79" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1075,7 @@
       <c r="BQ1" s="7"/>
       <c r="BR1" s="8"/>
     </row>
-    <row r="2" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1101,7 @@
       <c r="BQ2" s="10"/>
       <c r="BR2" s="11"/>
     </row>
-    <row r="3" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1266,7 +1192,7 @@
       <c r="BZ3" s="4"/>
       <c r="CA3" s="4"/>
     </row>
-    <row r="4" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1289,7 +1215,7 @@
       <c r="BQ4" s="10"/>
       <c r="BR4" s="11"/>
     </row>
-    <row r="5" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1311,7 +1237,7 @@
       <c r="BQ5" s="10"/>
       <c r="BR5" s="11"/>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="15" t="s">
         <v>1</v>
       </c>
@@ -1416,7 +1342,7 @@
       <c r="BZ6" s="18"/>
       <c r="CA6" s="18"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="15" t="s">
         <v>5</v>
       </c>
@@ -1426,15 +1352,15 @@
       <c r="C7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="24" t="n">
-        <f aca="false">IF(C6=D6,C7+1,1)</f>
+      <c r="D7" s="24">
+        <f>IF(C6=D6,C7+1,1)</f>
         <v>1</v>
       </c>
-      <c r="E7" s="24" t="n">
-        <f aca="false">IF(D6=E6,D7+1,1)</f>
+      <c r="E7" s="24">
+        <f>IF(D6=E6,D7+1,1)</f>
         <v>2</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F7" s="24">
         <v>3</v>
       </c>
       <c r="G7" s="24" t="s">
@@ -1523,7 +1449,7 @@
       <c r="BZ7" s="25"/>
       <c r="CA7" s="25"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="31" t="s">
         <v>14</v>
       </c>
@@ -1531,31 +1457,31 @@
         <v>15</v>
       </c>
       <c r="C8" s="32"/>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="33">
         <v>70</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="34">
         <v>70</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="34">
         <v>70</v>
       </c>
-      <c r="G8" s="34" t="n">
+      <c r="G8" s="34">
         <v>70</v>
       </c>
-      <c r="H8" s="34" t="n">
+      <c r="H8" s="34">
         <v>70</v>
       </c>
-      <c r="I8" s="34" t="n">
+      <c r="I8" s="34">
         <v>70</v>
       </c>
-      <c r="J8" s="34" t="n">
+      <c r="J8" s="34">
         <v>70</v>
       </c>
-      <c r="K8" s="34" t="n">
+      <c r="K8" s="34">
         <v>70</v>
       </c>
-      <c r="L8" s="34" t="n">
+      <c r="L8" s="34">
         <v>70</v>
       </c>
       <c r="M8" s="35"/>
@@ -1626,7 +1552,7 @@
       <c r="BZ8" s="35"/>
       <c r="CA8" s="35"/>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="31" t="s">
         <v>16</v>
       </c>
@@ -1634,31 +1560,31 @@
         <v>17</v>
       </c>
       <c r="C9" s="32"/>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="34">
         <v>75</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="34">
         <v>75</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="34">
         <v>75</v>
       </c>
-      <c r="G9" s="34" t="n">
+      <c r="G9" s="34">
         <v>75</v>
       </c>
-      <c r="H9" s="34" t="n">
+      <c r="H9" s="34">
         <v>75</v>
       </c>
-      <c r="I9" s="34" t="n">
+      <c r="I9" s="34">
         <v>75</v>
       </c>
-      <c r="J9" s="34" t="n">
+      <c r="J9" s="34">
         <v>75</v>
       </c>
-      <c r="K9" s="34" t="n">
+      <c r="K9" s="34">
         <v>75</v>
       </c>
-      <c r="L9" s="34" t="n">
+      <c r="L9" s="34">
         <v>75</v>
       </c>
       <c r="M9" s="35"/>
@@ -1729,7 +1655,7 @@
       <c r="BZ9" s="35"/>
       <c r="CA9" s="35"/>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="31" t="s">
         <v>18</v>
       </c>
@@ -1737,31 +1663,31 @@
         <v>19</v>
       </c>
       <c r="C10" s="38"/>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="34">
         <v>60</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="34">
         <v>60</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="34">
         <v>60</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G10" s="34">
         <v>60</v>
       </c>
-      <c r="H10" s="34" t="n">
+      <c r="H10" s="34">
         <v>60</v>
       </c>
-      <c r="I10" s="34" t="n">
+      <c r="I10" s="34">
         <v>60</v>
       </c>
-      <c r="J10" s="34" t="n">
+      <c r="J10" s="34">
         <v>60</v>
       </c>
-      <c r="K10" s="34" t="n">
+      <c r="K10" s="34">
         <v>60</v>
       </c>
-      <c r="L10" s="34" t="n">
+      <c r="L10" s="34">
         <v>60</v>
       </c>
       <c r="M10" s="35"/>
@@ -1832,7 +1758,7 @@
       <c r="BZ10" s="35"/>
       <c r="CA10" s="35"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="31" t="s">
         <v>20</v>
       </c>
@@ -1840,31 +1766,31 @@
         <v>21</v>
       </c>
       <c r="C11" s="38"/>
-      <c r="D11" s="34" t="n">
+      <c r="D11" s="34">
         <v>90</v>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="34">
         <v>90</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="34">
         <v>90</v>
       </c>
-      <c r="G11" s="34" t="n">
+      <c r="G11" s="34">
         <v>90</v>
       </c>
-      <c r="H11" s="34" t="n">
+      <c r="H11" s="34">
         <v>90</v>
       </c>
-      <c r="I11" s="34" t="n">
+      <c r="I11" s="34">
         <v>90</v>
       </c>
-      <c r="J11" s="34" t="n">
+      <c r="J11" s="34">
         <v>90</v>
       </c>
-      <c r="K11" s="34" t="n">
+      <c r="K11" s="34">
         <v>90</v>
       </c>
-      <c r="L11" s="34" t="n">
+      <c r="L11" s="34">
         <v>90</v>
       </c>
       <c r="M11" s="35"/>
@@ -1935,7 +1861,7 @@
       <c r="BZ11" s="35"/>
       <c r="CA11" s="35"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="31" t="s">
         <v>22</v>
       </c>
@@ -1943,31 +1869,31 @@
         <v>23</v>
       </c>
       <c r="C12" s="32"/>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="34">
         <v>1000</v>
       </c>
-      <c r="E12" s="34" t="n">
+      <c r="E12" s="34">
         <v>1000</v>
       </c>
       <c r="F12" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="G12" s="34" t="n">
+      <c r="G12" s="34">
         <v>1000</v>
       </c>
-      <c r="H12" s="34" t="n">
+      <c r="H12" s="34">
         <v>1000</v>
       </c>
-      <c r="I12" s="34" t="n">
+      <c r="I12" s="34">
         <v>1000</v>
       </c>
-      <c r="J12" s="34" t="n">
+      <c r="J12" s="34">
         <v>1000</v>
       </c>
-      <c r="K12" s="34" t="n">
+      <c r="K12" s="34">
         <v>1000</v>
       </c>
-      <c r="L12" s="34" t="n">
+      <c r="L12" s="34">
         <v>1000</v>
       </c>
       <c r="M12" s="35"/>
@@ -2038,7 +1964,7 @@
       <c r="BZ12" s="35"/>
       <c r="CA12" s="35"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="31" t="s">
         <v>25</v>
       </c>
@@ -2046,7 +1972,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="38"/>
-      <c r="D13" s="34" t="n">
+      <c r="D13" s="34">
         <v>500</v>
       </c>
       <c r="E13" s="34" t="s">
@@ -2055,22 +1981,22 @@
       <c r="F13" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="34" t="n">
+      <c r="G13" s="34">
         <v>500</v>
       </c>
-      <c r="H13" s="34" t="n">
+      <c r="H13" s="34">
         <v>500</v>
       </c>
-      <c r="I13" s="34" t="n">
+      <c r="I13" s="34">
         <v>500</v>
       </c>
-      <c r="J13" s="34" t="n">
+      <c r="J13" s="34">
         <v>500</v>
       </c>
-      <c r="K13" s="34" t="n">
+      <c r="K13" s="34">
         <v>500</v>
       </c>
-      <c r="L13" s="34" t="n">
+      <c r="L13" s="34">
         <v>500</v>
       </c>
       <c r="M13" s="35"/>
@@ -2141,7 +2067,7 @@
       <c r="BZ13" s="35"/>
       <c r="CA13" s="35"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="31" t="s">
         <v>29</v>
       </c>
@@ -2149,31 +2075,31 @@
         <v>30</v>
       </c>
       <c r="C14" s="38"/>
-      <c r="D14" s="34" t="n">
+      <c r="D14" s="34">
         <v>100</v>
       </c>
       <c r="E14" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="34" t="n">
+      <c r="F14" s="34">
         <v>100</v>
       </c>
-      <c r="G14" s="34" t="n">
+      <c r="G14" s="34">
         <v>100</v>
       </c>
-      <c r="H14" s="34" t="n">
+      <c r="H14" s="34">
         <v>100</v>
       </c>
-      <c r="I14" s="34" t="n">
+      <c r="I14" s="34">
         <v>100</v>
       </c>
-      <c r="J14" s="34" t="n">
+      <c r="J14" s="34">
         <v>100</v>
       </c>
-      <c r="K14" s="34" t="n">
+      <c r="K14" s="34">
         <v>100</v>
       </c>
-      <c r="L14" s="34" t="n">
+      <c r="L14" s="34">
         <v>100</v>
       </c>
       <c r="M14" s="35"/>
@@ -2244,7 +2170,7 @@
       <c r="BZ14" s="35"/>
       <c r="CA14" s="35"/>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="31" t="s">
         <v>32</v>
       </c>
@@ -2252,31 +2178,31 @@
         <v>33</v>
       </c>
       <c r="C15" s="38"/>
-      <c r="D15" s="34" t="n">
+      <c r="D15" s="34">
         <v>200</v>
       </c>
       <c r="E15" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="34" t="n">
+      <c r="F15" s="34">
         <v>200</v>
       </c>
-      <c r="G15" s="34" t="n">
+      <c r="G15" s="34">
         <v>200</v>
       </c>
-      <c r="H15" s="34" t="n">
+      <c r="H15" s="34">
         <v>200</v>
       </c>
-      <c r="I15" s="34" t="n">
+      <c r="I15" s="34">
         <v>200</v>
       </c>
-      <c r="J15" s="34" t="n">
+      <c r="J15" s="34">
         <v>200</v>
       </c>
-      <c r="K15" s="34" t="n">
+      <c r="K15" s="34">
         <v>200</v>
       </c>
-      <c r="L15" s="34" t="n">
+      <c r="L15" s="34">
         <v>200</v>
       </c>
       <c r="M15" s="35"/>
@@ -2347,7 +2273,7 @@
       <c r="BZ15" s="35"/>
       <c r="CA15" s="35"/>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="31" t="s">
         <v>35</v>
       </c>
@@ -2355,7 +2281,7 @@
         <v>36</v>
       </c>
       <c r="C16" s="38"/>
-      <c r="D16" s="34" t="n">
+      <c r="D16" s="34">
         <v>120</v>
       </c>
       <c r="E16" s="34" t="s">
@@ -2364,22 +2290,22 @@
       <c r="F16" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="G16" s="34" t="n">
+      <c r="G16" s="34">
         <v>120</v>
       </c>
-      <c r="H16" s="34" t="n">
+      <c r="H16" s="34">
         <v>120</v>
       </c>
-      <c r="I16" s="34" t="n">
+      <c r="I16" s="34">
         <v>120</v>
       </c>
-      <c r="J16" s="34" t="n">
+      <c r="J16" s="34">
         <v>120</v>
       </c>
-      <c r="K16" s="34" t="n">
+      <c r="K16" s="34">
         <v>120</v>
       </c>
-      <c r="L16" s="34" t="n">
+      <c r="L16" s="34">
         <v>120</v>
       </c>
       <c r="M16" s="35"/>
@@ -2450,7 +2376,7 @@
       <c r="BZ16" s="35"/>
       <c r="CA16" s="35"/>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="31" t="s">
         <v>39</v>
       </c>
@@ -2458,7 +2384,7 @@
         <v>40</v>
       </c>
       <c r="C17" s="32"/>
-      <c r="D17" s="34" t="n">
+      <c r="D17" s="34">
         <v>20</v>
       </c>
       <c r="E17" s="34" t="s">
@@ -2467,22 +2393,22 @@
       <c r="F17" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="G17" s="34" t="n">
+      <c r="G17" s="34">
         <v>20</v>
       </c>
-      <c r="H17" s="34" t="n">
+      <c r="H17" s="34">
         <v>20</v>
       </c>
-      <c r="I17" s="34" t="n">
+      <c r="I17" s="34">
         <v>20</v>
       </c>
-      <c r="J17" s="34" t="n">
+      <c r="J17" s="34">
         <v>20</v>
       </c>
-      <c r="K17" s="34" t="n">
+      <c r="K17" s="34">
         <v>20</v>
       </c>
-      <c r="L17" s="34" t="n">
+      <c r="L17" s="34">
         <v>20</v>
       </c>
       <c r="M17" s="35"/>
@@ -2553,7 +2479,7 @@
       <c r="BZ17" s="35"/>
       <c r="CA17" s="35"/>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="31" t="s">
         <v>43</v>
       </c>
@@ -2656,7 +2582,7 @@
       <c r="BZ18" s="35"/>
       <c r="CA18" s="35"/>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="31" t="s">
         <v>48</v>
       </c>
@@ -2664,31 +2590,31 @@
         <v>49</v>
       </c>
       <c r="C19" s="32"/>
-      <c r="D19" s="34" t="n">
+      <c r="D19" s="34">
         <v>150</v>
       </c>
       <c r="E19" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="34">
         <v>150</v>
       </c>
-      <c r="G19" s="34" t="n">
+      <c r="G19" s="34">
         <v>150</v>
       </c>
-      <c r="H19" s="34" t="n">
+      <c r="H19" s="34">
         <v>150</v>
       </c>
-      <c r="I19" s="34" t="n">
+      <c r="I19" s="34">
         <v>150</v>
       </c>
-      <c r="J19" s="34" t="n">
+      <c r="J19" s="34">
         <v>150</v>
       </c>
-      <c r="K19" s="34" t="n">
+      <c r="K19" s="34">
         <v>150</v>
       </c>
-      <c r="L19" s="34" t="n">
+      <c r="L19" s="34">
         <v>150</v>
       </c>
       <c r="M19" s="35"/>
@@ -2759,7 +2685,7 @@
       <c r="BZ19" s="35"/>
       <c r="CA19" s="35"/>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="31" t="s">
         <v>51</v>
       </c>
@@ -2767,31 +2693,31 @@
         <v>52</v>
       </c>
       <c r="C20" s="32"/>
-      <c r="D20" s="34" t="n">
+      <c r="D20" s="34">
         <v>55</v>
       </c>
       <c r="E20" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="F20" s="34" t="n">
+      <c r="F20" s="34">
         <v>55</v>
       </c>
-      <c r="G20" s="34" t="n">
+      <c r="G20" s="34">
         <v>55</v>
       </c>
-      <c r="H20" s="34" t="n">
+      <c r="H20" s="34">
         <v>55</v>
       </c>
-      <c r="I20" s="34" t="n">
+      <c r="I20" s="34">
         <v>55</v>
       </c>
-      <c r="J20" s="34" t="n">
+      <c r="J20" s="34">
         <v>55</v>
       </c>
-      <c r="K20" s="34" t="n">
+      <c r="K20" s="34">
         <v>55</v>
       </c>
-      <c r="L20" s="34" t="n">
+      <c r="L20" s="34">
         <v>55</v>
       </c>
       <c r="M20" s="35"/>
@@ -2862,7 +2788,7 @@
       <c r="BZ20" s="35"/>
       <c r="CA20" s="35"/>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="31" t="s">
         <v>54</v>
       </c>
@@ -2870,31 +2796,31 @@
         <v>55</v>
       </c>
       <c r="C21" s="38"/>
-      <c r="D21" s="34" t="n">
+      <c r="D21" s="34">
         <v>72</v>
       </c>
       <c r="E21" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="F21" s="34" t="n">
+      <c r="F21" s="34">
         <v>72</v>
       </c>
-      <c r="G21" s="34" t="n">
+      <c r="G21" s="34">
         <v>72</v>
       </c>
-      <c r="H21" s="34" t="n">
+      <c r="H21" s="34">
         <v>72</v>
       </c>
-      <c r="I21" s="34" t="n">
+      <c r="I21" s="34">
         <v>72</v>
       </c>
-      <c r="J21" s="34" t="n">
+      <c r="J21" s="34">
         <v>72</v>
       </c>
-      <c r="K21" s="34" t="n">
+      <c r="K21" s="34">
         <v>72</v>
       </c>
-      <c r="L21" s="34" t="n">
+      <c r="L21" s="34">
         <v>72</v>
       </c>
       <c r="M21" s="35"/>
@@ -2965,7 +2891,7 @@
       <c r="BZ21" s="35"/>
       <c r="CA21" s="35"/>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="31" t="s">
         <v>57</v>
       </c>
@@ -2973,31 +2899,31 @@
         <v>58</v>
       </c>
       <c r="C22" s="38"/>
-      <c r="D22" s="34" t="n">
+      <c r="D22" s="34">
         <v>400</v>
       </c>
       <c r="E22" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="F22" s="34" t="n">
+      <c r="F22" s="34">
         <v>400</v>
       </c>
-      <c r="G22" s="34" t="n">
+      <c r="G22" s="34">
         <v>400</v>
       </c>
-      <c r="H22" s="34" t="n">
+      <c r="H22" s="34">
         <v>400</v>
       </c>
-      <c r="I22" s="34" t="n">
+      <c r="I22" s="34">
         <v>400</v>
       </c>
-      <c r="J22" s="34" t="n">
+      <c r="J22" s="34">
         <v>400</v>
       </c>
-      <c r="K22" s="34" t="n">
+      <c r="K22" s="34">
         <v>400</v>
       </c>
-      <c r="L22" s="34" t="n">
+      <c r="L22" s="34">
         <v>400</v>
       </c>
       <c r="M22" s="35"/>
@@ -3068,7 +2994,7 @@
       <c r="BZ22" s="35"/>
       <c r="CA22" s="35"/>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="31" t="s">
         <v>60</v>
       </c>
@@ -3171,7 +3097,7 @@
       <c r="BZ23" s="35"/>
       <c r="CA23" s="35"/>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="31" t="s">
         <v>64</v>
       </c>
@@ -3274,7 +3200,7 @@
       <c r="BZ24" s="35"/>
       <c r="CA24" s="35"/>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="31" t="s">
         <v>68</v>
       </c>
@@ -3282,31 +3208,31 @@
         <v>69</v>
       </c>
       <c r="C25" s="38"/>
-      <c r="D25" s="34" t="n">
+      <c r="D25" s="34">
         <v>1</v>
       </c>
       <c r="E25" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="F25" s="34" t="n">
+      <c r="F25" s="34">
         <v>1</v>
       </c>
-      <c r="G25" s="34" t="n">
+      <c r="G25" s="34">
         <v>1</v>
       </c>
-      <c r="H25" s="34" t="n">
+      <c r="H25" s="34">
         <v>1</v>
       </c>
-      <c r="I25" s="34" t="n">
+      <c r="I25" s="34">
         <v>1</v>
       </c>
-      <c r="J25" s="34" t="n">
+      <c r="J25" s="34">
         <v>1</v>
       </c>
-      <c r="K25" s="34" t="n">
+      <c r="K25" s="34">
         <v>1</v>
       </c>
-      <c r="L25" s="34" t="n">
+      <c r="L25" s="34">
         <v>1</v>
       </c>
       <c r="M25" s="35"/>
@@ -3377,7 +3303,7 @@
       <c r="BZ25" s="35"/>
       <c r="CA25" s="35"/>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="31" t="s">
         <v>71</v>
       </c>
@@ -3385,31 +3311,31 @@
         <v>72</v>
       </c>
       <c r="C26" s="38"/>
-      <c r="D26" s="34" t="n">
+      <c r="D26" s="34">
         <v>1</v>
       </c>
       <c r="E26" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="34" t="n">
+      <c r="F26" s="34">
         <v>1</v>
       </c>
-      <c r="G26" s="34" t="n">
+      <c r="G26" s="34">
         <v>1</v>
       </c>
-      <c r="H26" s="34" t="n">
+      <c r="H26" s="34">
         <v>1</v>
       </c>
-      <c r="I26" s="34" t="n">
+      <c r="I26" s="34">
         <v>1</v>
       </c>
-      <c r="J26" s="34" t="n">
+      <c r="J26" s="34">
         <v>1</v>
       </c>
-      <c r="K26" s="34" t="n">
+      <c r="K26" s="34">
         <v>1</v>
       </c>
-      <c r="L26" s="34" t="n">
+      <c r="L26" s="34">
         <v>1</v>
       </c>
       <c r="M26" s="35"/>
@@ -3480,7 +3406,7 @@
       <c r="BZ26" s="35"/>
       <c r="CA26" s="35"/>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="31" t="s">
         <v>74</v>
       </c>
@@ -3488,31 +3414,31 @@
         <v>75</v>
       </c>
       <c r="C27" s="32"/>
-      <c r="D27" s="34" t="n">
+      <c r="D27" s="34">
         <v>1</v>
       </c>
       <c r="E27" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F27" s="34" t="n">
+      <c r="F27" s="34">
         <v>1</v>
       </c>
-      <c r="G27" s="34" t="n">
+      <c r="G27" s="34">
         <v>1</v>
       </c>
-      <c r="H27" s="34" t="n">
+      <c r="H27" s="34">
         <v>1</v>
       </c>
-      <c r="I27" s="34" t="n">
+      <c r="I27" s="34">
         <v>1</v>
       </c>
-      <c r="J27" s="34" t="n">
+      <c r="J27" s="34">
         <v>1</v>
       </c>
-      <c r="K27" s="34" t="n">
+      <c r="K27" s="34">
         <v>1</v>
       </c>
-      <c r="L27" s="34" t="n">
+      <c r="L27" s="34">
         <v>1</v>
       </c>
       <c r="M27" s="35"/>
@@ -3583,7 +3509,7 @@
       <c r="BZ27" s="35"/>
       <c r="CA27" s="35"/>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="31" t="s">
         <v>77</v>
       </c>
@@ -3591,31 +3517,31 @@
         <v>78</v>
       </c>
       <c r="C28" s="32"/>
-      <c r="D28" s="34" t="n">
+      <c r="D28" s="34">
         <v>1</v>
       </c>
       <c r="E28" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="F28" s="34" t="n">
+      <c r="F28" s="34">
         <v>1</v>
       </c>
-      <c r="G28" s="34" t="n">
+      <c r="G28" s="34">
         <v>1</v>
       </c>
-      <c r="H28" s="34" t="n">
+      <c r="H28" s="34">
         <v>1</v>
       </c>
-      <c r="I28" s="34" t="n">
+      <c r="I28" s="34">
         <v>1</v>
       </c>
-      <c r="J28" s="34" t="n">
+      <c r="J28" s="34">
         <v>1</v>
       </c>
-      <c r="K28" s="34" t="n">
+      <c r="K28" s="34">
         <v>1</v>
       </c>
-      <c r="L28" s="34" t="n">
+      <c r="L28" s="34">
         <v>1</v>
       </c>
       <c r="M28" s="35"/>
@@ -3686,7 +3612,7 @@
       <c r="BZ28" s="35"/>
       <c r="CA28" s="35"/>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="31" t="s">
         <v>80</v>
       </c>
@@ -3789,7 +3715,7 @@
       <c r="BZ29" s="35"/>
       <c r="CA29" s="35"/>
     </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="31" t="s">
         <v>83</v>
       </c>
@@ -3797,10 +3723,10 @@
         <v>84</v>
       </c>
       <c r="C30" s="38"/>
-      <c r="D30" s="34" t="n">
+      <c r="D30" s="34">
         <v>50</v>
       </c>
-      <c r="E30" s="34" t="n">
+      <c r="E30" s="34">
         <v>55</v>
       </c>
       <c r="F30" s="34" t="s">
@@ -3892,7 +3818,7 @@
       <c r="BZ30" s="35"/>
       <c r="CA30" s="35"/>
     </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="31" t="s">
         <v>86</v>
       </c>
@@ -3900,28 +3826,28 @@
         <v>87</v>
       </c>
       <c r="C31" s="38"/>
-      <c r="D31" s="34" t="n">
+      <c r="D31" s="34">
         <v>55</v>
       </c>
-      <c r="E31" s="34" t="n">
+      <c r="E31" s="34">
         <v>55</v>
       </c>
-      <c r="F31" s="34" t="n">
+      <c r="F31" s="34">
         <v>55</v>
       </c>
-      <c r="G31" s="34" t="n">
+      <c r="G31" s="34">
         <v>55</v>
       </c>
-      <c r="H31" s="34" t="n">
+      <c r="H31" s="34">
         <v>55</v>
       </c>
-      <c r="I31" s="34" t="n">
+      <c r="I31" s="34">
         <v>55</v>
       </c>
-      <c r="J31" s="34" t="n">
+      <c r="J31" s="34">
         <v>55</v>
       </c>
-      <c r="K31" s="34" t="n">
+      <c r="K31" s="34">
         <v>55</v>
       </c>
       <c r="L31" s="34" t="s">
@@ -3995,7 +3921,7 @@
       <c r="BZ31" s="35"/>
       <c r="CA31" s="35"/>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="31" t="s">
         <v>89</v>
       </c>
@@ -4098,7 +4024,7 @@
       <c r="BZ32" s="35"/>
       <c r="CA32" s="35"/>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="31" t="s">
         <v>91</v>
       </c>
@@ -4201,7 +4127,7 @@
       <c r="BZ33" s="35"/>
       <c r="CA33" s="35"/>
     </row>
-    <row r="34" s="41" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:79" s="41" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="39" t="s">
         <v>94</v>
       </c>
@@ -4227,7 +4153,7 @@
       <c r="BQ34" s="42"/>
       <c r="BR34" s="43"/>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="31" t="s">
         <v>96</v>
       </c>
@@ -4330,7 +4256,7 @@
       <c r="BZ35" s="44"/>
       <c r="CA35" s="44"/>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="47" t="s">
         <v>2</v>
       </c>
@@ -4425,7 +4351,7 @@
       <c r="BZ36" s="35"/>
       <c r="CA36" s="35"/>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="47" t="s">
         <v>103</v>
       </c>
@@ -4520,7 +4446,7 @@
       <c r="BZ37" s="35"/>
       <c r="CA37" s="35"/>
     </row>
-    <row r="38" s="41" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:79" s="41" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="39" t="s">
         <v>108</v>
       </c>
@@ -4548,41 +4474,41 @@
       <c r="BQ38" s="42"/>
       <c r="BR38" s="43"/>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="31" t="s">
         <v>14</v>
       </c>
       <c r="B39" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="C39" s="38" t="n">
+      <c r="C39" s="38">
         <v>0</v>
       </c>
       <c r="D39" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E39" s="33" t="n">
+      <c r="E39" s="33">
         <v>70</v>
       </c>
-      <c r="F39" s="34" t="n">
+      <c r="F39" s="34">
         <v>70</v>
       </c>
-      <c r="G39" s="34" t="n">
+      <c r="G39" s="34">
         <v>70</v>
       </c>
-      <c r="H39" s="34" t="n">
+      <c r="H39" s="34">
         <v>70</v>
       </c>
-      <c r="I39" s="34" t="n">
+      <c r="I39" s="34">
         <v>70</v>
       </c>
-      <c r="J39" s="34" t="n">
+      <c r="J39" s="34">
         <v>70</v>
       </c>
-      <c r="K39" s="34" t="n">
+      <c r="K39" s="34">
         <v>70</v>
       </c>
-      <c r="L39" s="34" t="n">
+      <c r="L39" s="34">
         <v>70</v>
       </c>
       <c r="M39" s="35"/>
@@ -4653,41 +4579,41 @@
       <c r="BZ39" s="35"/>
       <c r="CA39" s="35"/>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="31" t="s">
         <v>16</v>
       </c>
       <c r="B40" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C40" s="38" t="n">
+      <c r="C40" s="38">
         <v>0</v>
       </c>
       <c r="D40" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E40" s="33" t="n">
+      <c r="E40" s="33">
         <v>75</v>
       </c>
-      <c r="F40" s="34" t="n">
+      <c r="F40" s="34">
         <v>75</v>
       </c>
-      <c r="G40" s="34" t="n">
+      <c r="G40" s="34">
         <v>75</v>
       </c>
-      <c r="H40" s="34" t="n">
+      <c r="H40" s="34">
         <v>75</v>
       </c>
-      <c r="I40" s="34" t="n">
+      <c r="I40" s="34">
         <v>75</v>
       </c>
-      <c r="J40" s="34" t="n">
+      <c r="J40" s="34">
         <v>75</v>
       </c>
-      <c r="K40" s="34" t="n">
+      <c r="K40" s="34">
         <v>75</v>
       </c>
-      <c r="L40" s="34" t="n">
+      <c r="L40" s="34">
         <v>75</v>
       </c>
       <c r="M40" s="35"/>
@@ -4758,41 +4684,41 @@
       <c r="BZ40" s="35"/>
       <c r="CA40" s="35"/>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="31" t="s">
         <v>18</v>
       </c>
       <c r="B41" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="C41" s="38" t="n">
+      <c r="C41" s="38">
         <v>0</v>
       </c>
       <c r="D41" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E41" s="33" t="n">
+      <c r="E41" s="33">
         <v>60</v>
       </c>
-      <c r="F41" s="34" t="n">
+      <c r="F41" s="34">
         <v>60</v>
       </c>
-      <c r="G41" s="34" t="n">
+      <c r="G41" s="34">
         <v>60</v>
       </c>
-      <c r="H41" s="34" t="n">
+      <c r="H41" s="34">
         <v>60</v>
       </c>
-      <c r="I41" s="34" t="n">
+      <c r="I41" s="34">
         <v>60</v>
       </c>
-      <c r="J41" s="34" t="n">
+      <c r="J41" s="34">
         <v>60</v>
       </c>
-      <c r="K41" s="34" t="n">
+      <c r="K41" s="34">
         <v>60</v>
       </c>
-      <c r="L41" s="34" t="n">
+      <c r="L41" s="34">
         <v>60</v>
       </c>
       <c r="M41" s="35"/>
@@ -4863,41 +4789,41 @@
       <c r="BZ41" s="35"/>
       <c r="CA41" s="35"/>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="31" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="C42" s="38" t="n">
+      <c r="C42" s="38">
         <v>0</v>
       </c>
       <c r="D42" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E42" s="33" t="n">
+      <c r="E42" s="33">
         <v>90</v>
       </c>
-      <c r="F42" s="34" t="n">
+      <c r="F42" s="34">
         <v>90</v>
       </c>
-      <c r="G42" s="34" t="n">
+      <c r="G42" s="34">
         <v>90</v>
       </c>
-      <c r="H42" s="34" t="n">
+      <c r="H42" s="34">
         <v>90</v>
       </c>
-      <c r="I42" s="34" t="n">
+      <c r="I42" s="34">
         <v>90</v>
       </c>
-      <c r="J42" s="34" t="n">
+      <c r="J42" s="34">
         <v>90</v>
       </c>
-      <c r="K42" s="34" t="n">
+      <c r="K42" s="34">
         <v>90</v>
       </c>
-      <c r="L42" s="34" t="n">
+      <c r="L42" s="34">
         <v>90</v>
       </c>
       <c r="M42" s="35"/>
@@ -4968,41 +4894,41 @@
       <c r="BZ42" s="35"/>
       <c r="CA42" s="35"/>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="31" t="s">
         <v>22</v>
       </c>
       <c r="B43" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="C43" s="38" t="n">
+      <c r="C43" s="38">
         <v>0</v>
       </c>
       <c r="D43" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E43" s="33" t="n">
+      <c r="E43" s="33">
         <v>1000</v>
       </c>
-      <c r="F43" s="34" t="n">
+      <c r="F43" s="34">
         <v>1000</v>
       </c>
-      <c r="G43" s="34" t="n">
+      <c r="G43" s="34">
         <v>1000</v>
       </c>
-      <c r="H43" s="34" t="n">
+      <c r="H43" s="34">
         <v>1000</v>
       </c>
-      <c r="I43" s="34" t="n">
+      <c r="I43" s="34">
         <v>1000</v>
       </c>
-      <c r="J43" s="34" t="n">
+      <c r="J43" s="34">
         <v>1000</v>
       </c>
-      <c r="K43" s="34" t="n">
+      <c r="K43" s="34">
         <v>1000</v>
       </c>
-      <c r="L43" s="34" t="n">
+      <c r="L43" s="34">
         <v>1000</v>
       </c>
       <c r="M43" s="35"/>
@@ -5073,41 +4999,41 @@
       <c r="BZ43" s="35"/>
       <c r="CA43" s="35"/>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="31" t="s">
         <v>25</v>
       </c>
       <c r="B44" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="C44" s="38" t="n">
+      <c r="C44" s="38">
         <v>0</v>
       </c>
       <c r="D44" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E44" s="33" t="n">
+      <c r="E44" s="33">
         <v>75</v>
       </c>
-      <c r="F44" s="34" t="n">
+      <c r="F44" s="34">
         <v>500</v>
       </c>
-      <c r="G44" s="34" t="n">
+      <c r="G44" s="34">
         <v>500</v>
       </c>
-      <c r="H44" s="34" t="n">
+      <c r="H44" s="34">
         <v>500</v>
       </c>
-      <c r="I44" s="34" t="n">
+      <c r="I44" s="34">
         <v>500</v>
       </c>
-      <c r="J44" s="34" t="n">
+      <c r="J44" s="34">
         <v>500</v>
       </c>
-      <c r="K44" s="34" t="n">
+      <c r="K44" s="34">
         <v>500</v>
       </c>
-      <c r="L44" s="34" t="n">
+      <c r="L44" s="34">
         <v>500</v>
       </c>
       <c r="M44" s="35"/>
@@ -5178,41 +5104,41 @@
       <c r="BZ44" s="35"/>
       <c r="CA44" s="35"/>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="31" t="s">
         <v>29</v>
       </c>
       <c r="B45" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="C45" s="38" t="n">
+      <c r="C45" s="38">
         <v>0</v>
       </c>
       <c r="D45" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E45" s="48" t="n">
+      <c r="E45" s="35">
         <v>150</v>
       </c>
-      <c r="F45" s="34" t="n">
+      <c r="F45" s="34">
         <v>100</v>
       </c>
-      <c r="G45" s="34" t="n">
+      <c r="G45" s="34">
         <v>100</v>
       </c>
-      <c r="H45" s="34" t="n">
+      <c r="H45" s="34">
         <v>100</v>
       </c>
-      <c r="I45" s="34" t="n">
+      <c r="I45" s="34">
         <v>100</v>
       </c>
-      <c r="J45" s="34" t="n">
+      <c r="J45" s="34">
         <v>100</v>
       </c>
-      <c r="K45" s="34" t="n">
+      <c r="K45" s="34">
         <v>100</v>
       </c>
-      <c r="L45" s="34" t="n">
+      <c r="L45" s="34">
         <v>100</v>
       </c>
       <c r="M45" s="35"/>
@@ -5283,41 +5209,41 @@
       <c r="BZ45" s="35"/>
       <c r="CA45" s="35"/>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="31" t="s">
         <v>32</v>
       </c>
       <c r="B46" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="C46" s="38" t="n">
+      <c r="C46" s="38">
         <v>0</v>
       </c>
       <c r="D46" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E46" s="33" t="n">
+      <c r="E46" s="33">
         <v>72</v>
       </c>
-      <c r="F46" s="34" t="n">
+      <c r="F46" s="34">
         <v>200</v>
       </c>
-      <c r="G46" s="34" t="n">
+      <c r="G46" s="34">
         <v>200</v>
       </c>
-      <c r="H46" s="34" t="n">
+      <c r="H46" s="34">
         <v>200</v>
       </c>
-      <c r="I46" s="34" t="n">
+      <c r="I46" s="34">
         <v>200</v>
       </c>
-      <c r="J46" s="34" t="n">
+      <c r="J46" s="34">
         <v>200</v>
       </c>
-      <c r="K46" s="34" t="n">
+      <c r="K46" s="34">
         <v>200</v>
       </c>
-      <c r="L46" s="34" t="n">
+      <c r="L46" s="34">
         <v>200</v>
       </c>
       <c r="M46" s="35"/>
@@ -5388,41 +5314,41 @@
       <c r="BZ46" s="35"/>
       <c r="CA46" s="35"/>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="31" t="s">
         <v>35</v>
       </c>
       <c r="B47" s="31" t="s">
         <v>119</v>
       </c>
-      <c r="C47" s="38" t="n">
+      <c r="C47" s="38">
         <v>0</v>
       </c>
       <c r="D47" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E47" s="33" t="n">
+      <c r="E47" s="33">
         <v>65</v>
       </c>
-      <c r="F47" s="34" t="n">
+      <c r="F47" s="34">
         <v>120</v>
       </c>
-      <c r="G47" s="34" t="n">
+      <c r="G47" s="34">
         <v>120</v>
       </c>
-      <c r="H47" s="34" t="n">
+      <c r="H47" s="34">
         <v>120</v>
       </c>
-      <c r="I47" s="34" t="n">
+      <c r="I47" s="34">
         <v>120</v>
       </c>
-      <c r="J47" s="34" t="n">
+      <c r="J47" s="34">
         <v>120</v>
       </c>
-      <c r="K47" s="34" t="n">
+      <c r="K47" s="34">
         <v>120</v>
       </c>
-      <c r="L47" s="34" t="n">
+      <c r="L47" s="34">
         <v>120</v>
       </c>
       <c r="M47" s="35"/>
@@ -5493,41 +5419,41 @@
       <c r="BZ47" s="35"/>
       <c r="CA47" s="35"/>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="31" t="s">
         <v>39</v>
       </c>
       <c r="B48" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="C48" s="38" t="n">
+      <c r="C48" s="38">
         <v>0</v>
       </c>
       <c r="D48" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E48" s="33" t="n">
+      <c r="E48" s="33">
         <v>68</v>
       </c>
-      <c r="F48" s="34" t="n">
+      <c r="F48" s="34">
         <v>20</v>
       </c>
-      <c r="G48" s="34" t="n">
+      <c r="G48" s="34">
         <v>20</v>
       </c>
-      <c r="H48" s="34" t="n">
+      <c r="H48" s="34">
         <v>20</v>
       </c>
-      <c r="I48" s="34" t="n">
+      <c r="I48" s="34">
         <v>20</v>
       </c>
-      <c r="J48" s="34" t="n">
+      <c r="J48" s="34">
         <v>20</v>
       </c>
-      <c r="K48" s="34" t="n">
+      <c r="K48" s="34">
         <v>20</v>
       </c>
-      <c r="L48" s="34" t="n">
+      <c r="L48" s="34">
         <v>20</v>
       </c>
       <c r="M48" s="35"/>
@@ -5598,41 +5524,41 @@
       <c r="BZ48" s="35"/>
       <c r="CA48" s="35"/>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="31" t="s">
         <v>43</v>
       </c>
       <c r="B49" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="C49" s="38" t="n">
+      <c r="C49" s="38">
         <v>0</v>
       </c>
       <c r="D49" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E49" s="33" t="n">
+      <c r="E49" s="33">
         <v>72</v>
       </c>
-      <c r="F49" s="34" t="n">
+      <c r="F49" s="34">
         <v>70</v>
       </c>
-      <c r="G49" s="34" t="n">
+      <c r="G49" s="34">
         <v>70</v>
       </c>
-      <c r="H49" s="34" t="n">
+      <c r="H49" s="34">
         <v>70</v>
       </c>
-      <c r="I49" s="34" t="n">
+      <c r="I49" s="34">
         <v>70</v>
       </c>
-      <c r="J49" s="34" t="n">
+      <c r="J49" s="34">
         <v>70</v>
       </c>
-      <c r="K49" s="34" t="n">
+      <c r="K49" s="34">
         <v>70</v>
       </c>
-      <c r="L49" s="34" t="n">
+      <c r="L49" s="34">
         <v>70</v>
       </c>
       <c r="M49" s="35"/>
@@ -5703,41 +5629,41 @@
       <c r="BZ49" s="35"/>
       <c r="CA49" s="35"/>
     </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="31" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="C50" s="38" t="n">
+      <c r="C50" s="38">
         <v>0</v>
       </c>
       <c r="D50" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E50" s="33" t="n">
+      <c r="E50" s="33">
         <v>72</v>
       </c>
-      <c r="F50" s="34" t="n">
+      <c r="F50" s="34">
         <v>150</v>
       </c>
-      <c r="G50" s="34" t="n">
+      <c r="G50" s="34">
         <v>150</v>
       </c>
-      <c r="H50" s="34" t="n">
+      <c r="H50" s="34">
         <v>150</v>
       </c>
-      <c r="I50" s="34" t="n">
+      <c r="I50" s="34">
         <v>150</v>
       </c>
-      <c r="J50" s="34" t="n">
+      <c r="J50" s="34">
         <v>150</v>
       </c>
-      <c r="K50" s="34" t="n">
+      <c r="K50" s="34">
         <v>150</v>
       </c>
-      <c r="L50" s="34" t="n">
+      <c r="L50" s="34">
         <v>150</v>
       </c>
       <c r="M50" s="35"/>
@@ -5808,14 +5734,14 @@
       <c r="BZ50" s="35"/>
       <c r="CA50" s="35"/>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="31" t="s">
         <v>51</v>
       </c>
       <c r="B51" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="C51" s="38" t="n">
+      <c r="C51" s="38">
         <v>0</v>
       </c>
       <c r="D51" s="33" t="s">
@@ -5824,25 +5750,25 @@
       <c r="E51" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="F51" s="34" t="n">
+      <c r="F51" s="34">
         <v>55</v>
       </c>
-      <c r="G51" s="34" t="n">
+      <c r="G51" s="34">
         <v>55</v>
       </c>
-      <c r="H51" s="34" t="n">
+      <c r="H51" s="34">
         <v>55</v>
       </c>
-      <c r="I51" s="34" t="n">
+      <c r="I51" s="34">
         <v>55</v>
       </c>
-      <c r="J51" s="34" t="n">
+      <c r="J51" s="34">
         <v>55</v>
       </c>
-      <c r="K51" s="34" t="n">
+      <c r="K51" s="34">
         <v>55</v>
       </c>
-      <c r="L51" s="34" t="n">
+      <c r="L51" s="34">
         <v>55</v>
       </c>
       <c r="M51" s="35"/>
@@ -5913,14 +5839,14 @@
       <c r="BZ51" s="35"/>
       <c r="CA51" s="35"/>
     </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="31" t="s">
         <v>54</v>
       </c>
       <c r="B52" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="C52" s="38" t="n">
+      <c r="C52" s="38">
         <v>0</v>
       </c>
       <c r="D52" s="33" t="s">
@@ -5929,25 +5855,25 @@
       <c r="E52" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="F52" s="34" t="n">
+      <c r="F52" s="34">
         <v>72</v>
       </c>
-      <c r="G52" s="34" t="n">
+      <c r="G52" s="34">
         <v>72</v>
       </c>
-      <c r="H52" s="34" t="n">
+      <c r="H52" s="34">
         <v>72</v>
       </c>
-      <c r="I52" s="34" t="n">
+      <c r="I52" s="34">
         <v>72</v>
       </c>
-      <c r="J52" s="34" t="n">
+      <c r="J52" s="34">
         <v>72</v>
       </c>
-      <c r="K52" s="34" t="n">
+      <c r="K52" s="34">
         <v>72</v>
       </c>
-      <c r="L52" s="34" t="n">
+      <c r="L52" s="34">
         <v>72</v>
       </c>
       <c r="M52" s="35"/>
@@ -6018,14 +5944,14 @@
       <c r="BZ52" s="35"/>
       <c r="CA52" s="35"/>
     </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="31" t="s">
         <v>57</v>
       </c>
       <c r="B53" s="31" t="s">
         <v>125</v>
       </c>
-      <c r="C53" s="38" t="n">
+      <c r="C53" s="38">
         <v>0</v>
       </c>
       <c r="D53" s="33" t="s">
@@ -6034,25 +5960,25 @@
       <c r="E53" s="33" t="s">
         <v>126</v>
       </c>
-      <c r="F53" s="34" t="n">
+      <c r="F53" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="G53" s="34">
         <v>400</v>
       </c>
-      <c r="G53" s="34" t="n">
+      <c r="H53" s="34">
         <v>400</v>
       </c>
-      <c r="H53" s="34" t="n">
+      <c r="I53" s="34">
         <v>400</v>
       </c>
-      <c r="I53" s="34" t="n">
+      <c r="J53" s="34">
         <v>400</v>
       </c>
-      <c r="J53" s="34" t="n">
+      <c r="K53" s="34">
         <v>400</v>
       </c>
-      <c r="K53" s="34" t="n">
-        <v>400</v>
-      </c>
-      <c r="L53" s="34" t="n">
+      <c r="L53" s="34">
         <v>400</v>
       </c>
       <c r="M53" s="35"/>
@@ -6123,14 +6049,14 @@
       <c r="BZ53" s="35"/>
       <c r="CA53" s="35"/>
     </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="31" t="s">
         <v>60</v>
       </c>
       <c r="B54" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="C54" s="38" t="n">
+      <c r="C54" s="38">
         <v>0</v>
       </c>
       <c r="D54" s="33" t="s">
@@ -6228,20 +6154,20 @@
       <c r="BZ54" s="35"/>
       <c r="CA54" s="35"/>
     </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="31" t="s">
         <v>64</v>
       </c>
       <c r="B55" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="C55" s="38" t="n">
+      <c r="C55" s="38">
         <v>0</v>
       </c>
       <c r="D55" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E55" s="33" t="n">
+      <c r="E55" s="33">
         <v>72</v>
       </c>
       <c r="F55" s="34" t="s">
@@ -6333,41 +6259,41 @@
       <c r="BZ55" s="35"/>
       <c r="CA55" s="35"/>
     </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="31" t="s">
         <v>68</v>
       </c>
       <c r="B56" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="C56" s="38" t="n">
+      <c r="C56" s="38">
         <v>0</v>
       </c>
       <c r="D56" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E56" s="33" t="n">
+      <c r="E56" s="33">
         <v>720</v>
       </c>
-      <c r="F56" s="34" t="n">
+      <c r="F56" s="34">
         <v>1</v>
       </c>
-      <c r="G56" s="34" t="n">
+      <c r="G56" s="34">
         <v>1</v>
       </c>
-      <c r="H56" s="34" t="n">
+      <c r="H56" s="34">
         <v>1</v>
       </c>
-      <c r="I56" s="34" t="n">
+      <c r="I56" s="34">
         <v>1</v>
       </c>
-      <c r="J56" s="34" t="n">
+      <c r="J56" s="34">
         <v>1</v>
       </c>
-      <c r="K56" s="34" t="n">
+      <c r="K56" s="34">
         <v>1</v>
       </c>
-      <c r="L56" s="34" t="n">
+      <c r="L56" s="34">
         <v>1</v>
       </c>
       <c r="M56" s="35"/>
@@ -6438,41 +6364,41 @@
       <c r="BZ56" s="35"/>
       <c r="CA56" s="35"/>
     </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="31" t="s">
         <v>71</v>
       </c>
       <c r="B57" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="C57" s="32" t="n">
+      <c r="C57" s="32">
         <v>0</v>
       </c>
       <c r="D57" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E57" s="33" t="n">
+      <c r="E57" s="33">
         <v>48</v>
       </c>
-      <c r="F57" s="34" t="n">
+      <c r="F57" s="34">
         <v>1</v>
       </c>
-      <c r="G57" s="34" t="n">
+      <c r="G57" s="34">
         <v>1</v>
       </c>
-      <c r="H57" s="34" t="n">
+      <c r="H57" s="34">
         <v>1</v>
       </c>
-      <c r="I57" s="34" t="n">
+      <c r="I57" s="34">
         <v>1</v>
       </c>
-      <c r="J57" s="34" t="n">
+      <c r="J57" s="34">
         <v>1</v>
       </c>
-      <c r="K57" s="34" t="n">
+      <c r="K57" s="34">
         <v>1</v>
       </c>
-      <c r="L57" s="34" t="n">
+      <c r="L57" s="34">
         <v>1</v>
       </c>
       <c r="M57" s="35"/>
@@ -6543,41 +6469,41 @@
       <c r="BZ57" s="35"/>
       <c r="CA57" s="35"/>
     </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="31" t="s">
         <v>74</v>
       </c>
       <c r="B58" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="C58" s="32" t="n">
+      <c r="C58" s="32">
         <v>0</v>
       </c>
       <c r="D58" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E58" s="33" t="n">
+      <c r="E58" s="33">
         <v>72</v>
       </c>
-      <c r="F58" s="34" t="n">
+      <c r="F58" s="34">
         <v>1</v>
       </c>
-      <c r="G58" s="34" t="n">
+      <c r="G58" s="34">
         <v>1</v>
       </c>
-      <c r="H58" s="34" t="n">
+      <c r="H58" s="34">
         <v>1</v>
       </c>
-      <c r="I58" s="34" t="n">
+      <c r="I58" s="34">
         <v>1</v>
       </c>
-      <c r="J58" s="34" t="n">
+      <c r="J58" s="34">
         <v>1</v>
       </c>
-      <c r="K58" s="34" t="n">
+      <c r="K58" s="34">
         <v>1</v>
       </c>
-      <c r="L58" s="34" t="n">
+      <c r="L58" s="34">
         <v>1</v>
       </c>
       <c r="M58" s="35"/>
@@ -6648,41 +6574,41 @@
       <c r="BZ58" s="35"/>
       <c r="CA58" s="35"/>
     </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="31" t="s">
         <v>77</v>
       </c>
       <c r="B59" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="C59" s="38" t="n">
+      <c r="C59" s="38">
         <v>0</v>
       </c>
       <c r="D59" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E59" s="33" t="n">
+      <c r="E59" s="33">
         <v>84</v>
       </c>
-      <c r="F59" s="34" t="n">
+      <c r="F59" s="34">
         <v>1</v>
       </c>
-      <c r="G59" s="34" t="n">
+      <c r="G59" s="34">
         <v>1</v>
       </c>
-      <c r="H59" s="34" t="n">
+      <c r="H59" s="34">
         <v>1</v>
       </c>
-      <c r="I59" s="34" t="n">
+      <c r="I59" s="34">
         <v>1</v>
       </c>
-      <c r="J59" s="34" t="n">
+      <c r="J59" s="34">
         <v>1</v>
       </c>
-      <c r="K59" s="34" t="n">
+      <c r="K59" s="34">
         <v>1</v>
       </c>
-      <c r="L59" s="34" t="n">
+      <c r="L59" s="34">
         <v>1</v>
       </c>
       <c r="M59" s="35"/>
@@ -6753,14 +6679,14 @@
       <c r="BZ59" s="35"/>
       <c r="CA59" s="35"/>
     </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="31" t="s">
         <v>83</v>
       </c>
       <c r="B60" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="C60" s="32" t="n">
+      <c r="C60" s="32">
         <v>0</v>
       </c>
       <c r="D60" s="33" t="s">
@@ -6769,25 +6695,25 @@
       <c r="E60" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="F60" s="34" t="n">
+      <c r="F60" s="34">
         <v>55</v>
       </c>
-      <c r="G60" s="34" t="n">
+      <c r="G60" s="34">
         <v>55</v>
       </c>
-      <c r="H60" s="34" t="n">
+      <c r="H60" s="34">
         <v>55</v>
       </c>
-      <c r="I60" s="34" t="n">
+      <c r="I60" s="34">
         <v>55</v>
       </c>
-      <c r="J60" s="34" t="n">
+      <c r="J60" s="34">
         <v>55</v>
       </c>
-      <c r="K60" s="34" t="n">
+      <c r="K60" s="34">
         <v>55</v>
       </c>
-      <c r="L60" s="34" t="n">
+      <c r="L60" s="34">
         <v>55</v>
       </c>
       <c r="M60" s="35"/>
@@ -6858,14 +6784,14 @@
       <c r="BZ60" s="35"/>
       <c r="CA60" s="35"/>
     </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" spans="1:79" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="31" t="s">
         <v>86</v>
       </c>
       <c r="B61" s="31" t="s">
         <v>135</v>
       </c>
-      <c r="C61" s="32" t="n">
+      <c r="C61" s="32">
         <v>0.05</v>
       </c>
       <c r="D61" s="33" t="s">
@@ -6874,22 +6800,22 @@
       <c r="E61" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="F61" s="34" t="n">
+      <c r="F61" s="34">
         <v>55</v>
       </c>
-      <c r="G61" s="34" t="n">
+      <c r="G61" s="34">
         <v>55</v>
       </c>
-      <c r="H61" s="34" t="n">
+      <c r="H61" s="34">
         <v>55</v>
       </c>
-      <c r="I61" s="34" t="n">
+      <c r="I61" s="34">
         <v>55</v>
       </c>
-      <c r="J61" s="34" t="n">
+      <c r="J61" s="34">
         <v>55</v>
       </c>
-      <c r="K61" s="34" t="n">
+      <c r="K61" s="34">
         <v>55</v>
       </c>
       <c r="L61" s="34" t="s">
@@ -6965,17 +6891,12 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="M8:ZZ33 M39:ZZ61">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>#ref!&lt;&gt;M8</formula>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>#REF!&lt;&gt;M8</formula>
     </cfRule>
   </conditionalFormatting>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Test for LAST and INTERPOLATE in expected output section separately
</commit_message>
<xml_diff>
--- a/tests/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
+++ b/tests/conformance_tests/foo/test_scripts/TestScript-foo.xlsx
@@ -1,33 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naqv776\Documents\Research\COPPER\copper_GitHub\issue52_handle_LAST_in_string_fxn\tests\conformance_tests\foo\test_scripts\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EEC7718-6583-435C-9F28-898E41FB990C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Script" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Script" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -36,12 +20,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="T5" authorId="0">
       <text>
         <r>
           <rPr>
@@ -49,14 +33,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     "1 total cooling requests remains at time data are recorded since loop output is still &gt;=85%" wording is unclear</t>
         </r>
       </text>
     </comment>
-    <comment ref="U5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="U5" authorId="0">
       <text>
         <r>
           <rPr>
@@ -64,14 +48,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     "0 total cooling requests remains at time data are recorded since loop output is &lt;85%" wording is unclear</t>
         </r>
       </text>
     </comment>
-    <comment ref="AI35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="AI35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -79,14 +63,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;70% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AJ35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="AJ35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -94,14 +78,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;70% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AM35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="AM35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -109,14 +93,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Needs to be increased.  Airflow needs to be &lt;50% of setpoint for 10 mins</t>
         </r>
       </text>
     </comment>
-    <comment ref="AW37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AW37" authorId="0">
       <text>
         <r>
           <rPr>
@@ -124,14 +108,14 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Unlikely that we will be able to get the loop to go to 50% exactly.  This needs to be an inequality</t>
         </r>
       </text>
     </comment>
-    <comment ref="BD37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="BC50" authorId="0">
       <text>
         <r>
           <rPr>
@@ -139,26 +123,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Possibility that the valve jumps above 94% and generates a request in this step
-Reply:
-    As noted, this is a concern that pops up repeatedly and we need to decide how we want to handle is.  See my other comment.
-Reply:
-    decision to leave unchanged for now</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BC50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     This can be simplified to AHUSupAirTempSp+MaxDeltaT since you already assumed heating loop will be 100% based on Vspt
@@ -176,438 +141,483 @@
         </r>
       </text>
     </comment>
+    <comment ref="BD37" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Possibility that the valve jumps above 94% and generates a request in this step
+Reply:
+    As noted, this is a concern that pops up repeatedly and we need to decide how we want to handle is.  See my other comment.
+Reply:
+    decision to leave unchanged for now</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="138">
-  <si>
-    <t>Dummy Test</t>
-  </si>
-  <si>
-    <t>Long Variable Name</t>
-  </si>
-  <si>
-    <t>Variable Name</t>
-  </si>
-  <si>
-    <t>Test Block</t>
-  </si>
-  <si>
-    <t>AA</t>
-  </si>
-  <si>
-    <t>Inputs</t>
-  </si>
-  <si>
-    <t>TestInputs</t>
-  </si>
-  <si>
-    <t>Test Step</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>ts_u1</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>ts_u2</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>ts_u3</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>ts_u4</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>ts_u5</t>
-  </si>
-  <si>
-    <t>=MULT(LAST;1)</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>ts_u6</t>
-  </si>
-  <si>
-    <t>=ts_u2</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 60; LAST; 500; 500; 500)</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>ts_u7</t>
-  </si>
-  <si>
-    <t>=RAMP(LAST; 200; 120; 10)</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>ts_u8</t>
-  </si>
-  <si>
-    <t>=ADD(60;12)</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>ts_u9</t>
-  </si>
-  <si>
-    <t>=MULT(5;13)</t>
-  </si>
-  <si>
-    <t>=ADD(LAST;55)</t>
-  </si>
-  <si>
-    <t>J</t>
-  </si>
-  <si>
-    <t>ts_u10</t>
-  </si>
-  <si>
-    <t>=SUB(72;4)</t>
-  </si>
-  <si>
-    <t>=SUB(LAST;48)</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>ts_u11</t>
-  </si>
-  <si>
-    <t>=RAMP(68; 72; 120; 10)</t>
-  </si>
-  <si>
-    <t>=RAMP(68; 72; 60; 10)</t>
-  </si>
-  <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>ts_u12</t>
-  </si>
-  <si>
-    <t>=RAMP(ts_u3; 72; 60; 10)</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>ts_u13</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90)</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>ts_u14</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73)</t>
-  </si>
-  <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>ts_u15</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73; 81)</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>ts_u16</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u3; 0; ts_u11; 70; 90; 73; 81)</t>
-  </si>
-  <si>
-    <t>Q</t>
-  </si>
-  <si>
-    <t>ts_u17</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>=ADD(ts_u3;12)</t>
-  </si>
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>ts_u18</t>
-  </si>
-  <si>
-    <t>=MULT(ts_u3;12)</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>ts_u19</t>
-  </si>
-  <si>
-    <t>=SUB(ts_u3;12)</t>
-  </si>
-  <si>
-    <t>T</t>
-  </si>
-  <si>
-    <t>ts_u20</t>
-  </si>
-  <si>
-    <t>=PERIODIC(ts_u11; 10)</t>
-  </si>
-  <si>
-    <t>U</t>
-  </si>
-  <si>
-    <t>ts_u21</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(ts_u1; 0; ts_u7; ADD(50; 20); 90)</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>ts_u22</t>
-  </si>
-  <si>
-    <t>ON</t>
-  </si>
-  <si>
-    <t>W</t>
-  </si>
-  <si>
-    <t>ts_u23</t>
-  </si>
-  <si>
-    <t>=LAST</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>ts_u24</t>
-  </si>
-  <si>
-    <t>55.04</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>ts_u25</t>
-  </si>
-  <si>
-    <t>Z</t>
-  </si>
-  <si>
-    <t>ts_u26</t>
-  </si>
-  <si>
-    <t>OCCUPIED</t>
-  </si>
-  <si>
-    <t>Conditions for Evaluation of Test Step</t>
-  </si>
-  <si>
-    <t>EvaluationConditions</t>
-  </si>
-  <si>
-    <t>Clock Time</t>
-  </si>
-  <si>
-    <t>ClockTime</t>
-  </si>
-  <si>
-    <t>0:00:30</t>
-  </si>
-  <si>
-    <t>0:01:00</t>
-  </si>
-  <si>
-    <t>VariableName</t>
-  </si>
-  <si>
-    <t>ts_y1</t>
-  </si>
-  <si>
-    <t>ts_y11</t>
-  </si>
-  <si>
-    <t>Variable Value</t>
-  </si>
-  <si>
-    <t>VariableValue</t>
-  </si>
-  <si>
-    <t>&gt;=69</t>
-  </si>
-  <si>
-    <t>&lt;=71</t>
-  </si>
-  <si>
-    <t>&gt;=70</t>
-  </si>
-  <si>
-    <t>Expected Outputs</t>
-  </si>
-  <si>
-    <t>TestOutputs</t>
-  </si>
-  <si>
-    <t>OutputTolerance</t>
-  </si>
-  <si>
-    <t>=ANY</t>
-  </si>
-  <si>
-    <t>ts_y2</t>
-  </si>
-  <si>
-    <t>ts_y3</t>
-  </si>
-  <si>
-    <t>ts_y4</t>
-  </si>
-  <si>
-    <t>ts_y5</t>
-  </si>
-  <si>
-    <t>ts_y6</t>
-  </si>
-  <si>
-    <t>ts_y7</t>
-  </si>
-  <si>
-    <t>ts_y8</t>
-  </si>
-  <si>
-    <t>ts_y9</t>
-  </si>
-  <si>
-    <t>ts_y10</t>
-  </si>
-  <si>
-    <t>ts_y12</t>
-  </si>
-  <si>
-    <t>ts_y13</t>
-  </si>
-  <si>
-    <t>82</t>
-  </si>
-  <si>
-    <t>ts_y14</t>
-  </si>
-  <si>
-    <t>ts_y15</t>
-  </si>
-  <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>ts_y16</t>
-  </si>
-  <si>
-    <t>ts_y17</t>
-  </si>
-  <si>
-    <t>ts_y18</t>
-  </si>
-  <si>
-    <t>ts_y19</t>
-  </si>
-  <si>
-    <t>ts_y20</t>
-  </si>
-  <si>
-    <t>ts_y21</t>
-  </si>
-  <si>
-    <t>ts_y23</t>
-  </si>
-  <si>
-    <t>&gt;50</t>
-  </si>
-  <si>
-    <t>ts_y24</t>
-  </si>
-  <si>
-    <t>&lt;56</t>
-  </si>
-  <si>
-    <t>=INTERPOLATE(LAST; 0; 162; 0; 800)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="140">
+  <si>
+    <t xml:space="preserve">Dummy Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long Variable Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestInputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(LAST;1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ts_u2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 60; LAST; 500; 500; 500)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(LAST; 200; 120; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(60;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(5;13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(LAST;55)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(72;4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(LAST;48)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(68; 72; 120; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(68; 72; 60; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=RAMP(ts_u3; 72; 60; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; 100; 70; 90; 73; 81)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u3; 0; ts_u11; 70; 90; 73; 81)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ADD(ts_u3;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=MULT(ts_u3;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUB(ts_u3;12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=PERIODIC(ts_u11; 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(ts_u1; 0; ts_u7; ADD(50; 20); 90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=LAST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">55.04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_u26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OCCUPIED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditions for Evaluation of Test Step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EvaluationConditions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clock Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ClockTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0:00:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0:01:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableValue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;=69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;=71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;=70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected Outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestOutputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OutputTolerance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=ANY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;LAST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;=LAST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=INTERPOLATE(81; 0; 162; 0; 800)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ts_y24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;56</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="h:mm:ss"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -617,7 +627,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -675,169 +685,258 @@
     </fill>
   </fills>
   <borders count="3">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
+      <right style="thick"/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thick">
-        <color auto="1"/>
-      </left>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thick"/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+  <cellXfs count="49">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -848,7 +947,6 @@
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -907,78 +1005,62 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="DejaVu Sans"/>
-        <a:cs typeface="DejaVu Sans"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="DejaVu Sans"/>
-        <a:cs typeface="DejaVu Sans"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1031,25 +1113,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ61"/>
-  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:CA61"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="64.15625" customWidth="1"/>
-    <col min="2" max="2" width="26.3125" customWidth="1"/>
-    <col min="3" max="3" width="18.47265625" customWidth="1"/>
-    <col min="4" max="6" width="50.68359375" style="1" customWidth="1"/>
-    <col min="7" max="79" width="50.68359375" style="2" customWidth="1"/>
-    <col min="80" max="1024" width="8.83984375" style="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="64.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="50.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="79" min="7" style="2" width="50.68"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="80" style="2" width="8.84"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" s="6" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1158,7 @@
       <c r="BQ1" s="7"/>
       <c r="BR1" s="8"/>
     </row>
-    <row r="2" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1101,7 +1184,7 @@
       <c r="BQ2" s="10"/>
       <c r="BR2" s="11"/>
     </row>
-    <row r="3" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1192,7 +1275,7 @@
       <c r="BZ3" s="4"/>
       <c r="CA3" s="4"/>
     </row>
-    <row r="4" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1298,7 @@
       <c r="BQ4" s="10"/>
       <c r="BR4" s="11"/>
     </row>
-    <row r="5" spans="1:79" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1237,7 +1320,7 @@
       <c r="BQ5" s="10"/>
       <c r="BR5" s="11"/>
     </row>
-    <row r="6" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
         <v>1</v>
       </c>
@@ -1342,7 +1425,7 @@
       <c r="BZ6" s="18"/>
       <c r="CA6" s="18"/>
     </row>
-    <row r="7" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
         <v>5</v>
       </c>
@@ -1352,15 +1435,15 @@
       <c r="C7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="24">
-        <f>IF(C6=D6,C7+1,1)</f>
+      <c r="D7" s="24" t="n">
+        <f aca="false">IF(C6=D6,C7+1,1)</f>
         <v>1</v>
       </c>
-      <c r="E7" s="24">
-        <f>IF(D6=E6,D7+1,1)</f>
+      <c r="E7" s="24" t="n">
+        <f aca="false">IF(D6=E6,D7+1,1)</f>
         <v>2</v>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="24" t="n">
         <v>3</v>
       </c>
       <c r="G7" s="24" t="s">
@@ -1449,7 +1532,7 @@
       <c r="BZ7" s="25"/>
       <c r="CA7" s="25"/>
     </row>
-    <row r="8" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
         <v>14</v>
       </c>
@@ -1457,31 +1540,31 @@
         <v>15</v>
       </c>
       <c r="C8" s="32"/>
-      <c r="D8" s="33">
+      <c r="D8" s="33" t="n">
         <v>70</v>
       </c>
-      <c r="E8" s="34">
+      <c r="E8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="F8" s="34">
+      <c r="F8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="H8" s="34">
+      <c r="H8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="L8" s="34">
+      <c r="L8" s="34" t="n">
         <v>70</v>
       </c>
       <c r="M8" s="35"/>
@@ -1552,7 +1635,7 @@
       <c r="BZ8" s="35"/>
       <c r="CA8" s="35"/>
     </row>
-    <row r="9" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
         <v>16</v>
       </c>
@@ -1560,31 +1643,31 @@
         <v>17</v>
       </c>
       <c r="C9" s="32"/>
-      <c r="D9" s="34">
+      <c r="D9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="E9" s="34">
+      <c r="E9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="F9" s="34">
+      <c r="F9" s="38" t="n">
+        <v>76</v>
+      </c>
+      <c r="G9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="G9" s="34">
+      <c r="H9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="H9" s="34">
+      <c r="I9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="I9" s="34">
+      <c r="J9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="J9" s="34">
+      <c r="K9" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="K9" s="34">
-        <v>75</v>
-      </c>
-      <c r="L9" s="34">
+      <c r="L9" s="34" t="n">
         <v>75</v>
       </c>
       <c r="M9" s="35"/>
@@ -1655,39 +1738,39 @@
       <c r="BZ9" s="35"/>
       <c r="CA9" s="35"/>
     </row>
-    <row r="10" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="38"/>
-      <c r="D10" s="34">
+      <c r="C10" s="39"/>
+      <c r="D10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="E10" s="34">
+      <c r="E10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="F10" s="34">
+      <c r="F10" s="38" t="n">
         <v>60</v>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="I10" s="34">
+      <c r="I10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="J10" s="34">
+      <c r="J10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="K10" s="34">
+      <c r="K10" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="L10" s="34">
+      <c r="L10" s="34" t="n">
         <v>60</v>
       </c>
       <c r="M10" s="35"/>
@@ -1758,39 +1841,39 @@
       <c r="BZ10" s="35"/>
       <c r="CA10" s="35"/>
     </row>
-    <row r="11" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="38"/>
-      <c r="D11" s="34">
+      <c r="C11" s="39"/>
+      <c r="D11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="E11" s="34">
+      <c r="E11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="F11" s="34">
+      <c r="F11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="H11" s="34">
+      <c r="H11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="I11" s="34">
+      <c r="I11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="J11" s="34">
+      <c r="J11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="K11" s="34">
+      <c r="K11" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="L11" s="34">
+      <c r="L11" s="34" t="n">
         <v>90</v>
       </c>
       <c r="M11" s="35"/>
@@ -1861,7 +1944,7 @@
       <c r="BZ11" s="35"/>
       <c r="CA11" s="35"/>
     </row>
-    <row r="12" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
         <v>22</v>
       </c>
@@ -1869,31 +1952,31 @@
         <v>23</v>
       </c>
       <c r="C12" s="32"/>
-      <c r="D12" s="34">
+      <c r="D12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="E12" s="34">
+      <c r="E12" s="34" t="n">
         <v>1000</v>
       </c>
       <c r="F12" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="G12" s="34">
+      <c r="G12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="I12" s="34">
+      <c r="I12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="J12" s="34">
+      <c r="J12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="K12" s="34">
+      <c r="K12" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="L12" s="34">
+      <c r="L12" s="34" t="n">
         <v>1000</v>
       </c>
       <c r="M12" s="35"/>
@@ -1964,15 +2047,15 @@
       <c r="BZ12" s="35"/>
       <c r="CA12" s="35"/>
     </row>
-    <row r="13" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
         <v>25</v>
       </c>
       <c r="B13" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="38"/>
-      <c r="D13" s="34">
+      <c r="C13" s="39"/>
+      <c r="D13" s="34" t="n">
         <v>500</v>
       </c>
       <c r="E13" s="34" t="s">
@@ -1981,22 +2064,22 @@
       <c r="F13" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="34">
+      <c r="G13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="H13" s="34">
+      <c r="H13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="I13" s="34">
+      <c r="I13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="J13" s="34">
+      <c r="J13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="K13" s="34">
+      <c r="K13" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="L13" s="34">
+      <c r="L13" s="34" t="n">
         <v>500</v>
       </c>
       <c r="M13" s="35"/>
@@ -2067,39 +2150,39 @@
       <c r="BZ13" s="35"/>
       <c r="CA13" s="35"/>
     </row>
-    <row r="14" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="s">
         <v>29</v>
       </c>
       <c r="B14" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="38"/>
-      <c r="D14" s="34">
+      <c r="C14" s="39"/>
+      <c r="D14" s="34" t="n">
         <v>100</v>
       </c>
       <c r="E14" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="34">
+      <c r="F14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="G14" s="34">
+      <c r="G14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="H14" s="34">
+      <c r="H14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="I14" s="34">
+      <c r="I14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="J14" s="34">
+      <c r="J14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="K14" s="34">
+      <c r="K14" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="L14" s="34">
+      <c r="L14" s="34" t="n">
         <v>100</v>
       </c>
       <c r="M14" s="35"/>
@@ -2170,39 +2253,39 @@
       <c r="BZ14" s="35"/>
       <c r="CA14" s="35"/>
     </row>
-    <row r="15" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="38"/>
-      <c r="D15" s="34">
+      <c r="C15" s="39"/>
+      <c r="D15" s="34" t="n">
         <v>200</v>
       </c>
       <c r="E15" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="34">
+      <c r="F15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="I15" s="34">
+      <c r="I15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="J15" s="34">
+      <c r="J15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="K15" s="34">
+      <c r="K15" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="L15" s="34">
+      <c r="L15" s="34" t="n">
         <v>200</v>
       </c>
       <c r="M15" s="35"/>
@@ -2273,15 +2356,15 @@
       <c r="BZ15" s="35"/>
       <c r="CA15" s="35"/>
     </row>
-    <row r="16" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
         <v>35</v>
       </c>
       <c r="B16" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="38"/>
-      <c r="D16" s="34">
+      <c r="C16" s="39"/>
+      <c r="D16" s="34" t="n">
         <v>120</v>
       </c>
       <c r="E16" s="34" t="s">
@@ -2290,22 +2373,22 @@
       <c r="F16" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="G16" s="34">
+      <c r="G16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="H16" s="34">
+      <c r="H16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="I16" s="34">
+      <c r="I16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="J16" s="34">
+      <c r="J16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="K16" s="34">
+      <c r="K16" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="L16" s="34">
+      <c r="L16" s="34" t="n">
         <v>120</v>
       </c>
       <c r="M16" s="35"/>
@@ -2376,7 +2459,7 @@
       <c r="BZ16" s="35"/>
       <c r="CA16" s="35"/>
     </row>
-    <row r="17" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="31" t="s">
         <v>39</v>
       </c>
@@ -2384,7 +2467,7 @@
         <v>40</v>
       </c>
       <c r="C17" s="32"/>
-      <c r="D17" s="34">
+      <c r="D17" s="34" t="n">
         <v>20</v>
       </c>
       <c r="E17" s="34" t="s">
@@ -2393,22 +2476,22 @@
       <c r="F17" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="G17" s="34">
+      <c r="G17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="H17" s="34">
+      <c r="H17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="I17" s="34">
+      <c r="I17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="J17" s="34">
+      <c r="J17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="K17" s="34">
+      <c r="K17" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="L17" s="34">
+      <c r="L17" s="34" t="n">
         <v>20</v>
       </c>
       <c r="M17" s="35"/>
@@ -2479,14 +2562,14 @@
       <c r="BZ17" s="35"/>
       <c r="CA17" s="35"/>
     </row>
-    <row r="18" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="31" t="s">
         <v>43</v>
       </c>
       <c r="B18" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="38"/>
+      <c r="C18" s="39"/>
       <c r="D18" s="34" t="s">
         <v>45</v>
       </c>
@@ -2582,7 +2665,7 @@
       <c r="BZ18" s="35"/>
       <c r="CA18" s="35"/>
     </row>
-    <row r="19" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="31" t="s">
         <v>48</v>
       </c>
@@ -2590,31 +2673,31 @@
         <v>49</v>
       </c>
       <c r="C19" s="32"/>
-      <c r="D19" s="34">
+      <c r="D19" s="34" t="n">
         <v>150</v>
       </c>
       <c r="E19" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="34">
+      <c r="F19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="G19" s="34">
+      <c r="G19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="H19" s="34">
+      <c r="H19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="I19" s="34">
+      <c r="I19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="J19" s="34">
+      <c r="J19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="K19" s="34">
+      <c r="K19" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="L19" s="34">
+      <c r="L19" s="34" t="n">
         <v>150</v>
       </c>
       <c r="M19" s="35"/>
@@ -2685,7 +2768,7 @@
       <c r="BZ19" s="35"/>
       <c r="CA19" s="35"/>
     </row>
-    <row r="20" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
         <v>51</v>
       </c>
@@ -2693,31 +2776,31 @@
         <v>52</v>
       </c>
       <c r="C20" s="32"/>
-      <c r="D20" s="34">
+      <c r="D20" s="34" t="n">
         <v>55</v>
       </c>
       <c r="E20" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="F20" s="34">
+      <c r="F20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G20" s="34">
+      <c r="G20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H20" s="34">
+      <c r="H20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I20" s="34">
+      <c r="I20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J20" s="34">
+      <c r="J20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K20" s="34">
+      <c r="K20" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="L20" s="34">
+      <c r="L20" s="34" t="n">
         <v>55</v>
       </c>
       <c r="M20" s="35"/>
@@ -2788,39 +2871,39 @@
       <c r="BZ20" s="35"/>
       <c r="CA20" s="35"/>
     </row>
-    <row r="21" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
         <v>54</v>
       </c>
       <c r="B21" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="38"/>
-      <c r="D21" s="34">
+      <c r="C21" s="39"/>
+      <c r="D21" s="34" t="n">
         <v>72</v>
       </c>
       <c r="E21" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="F21" s="34">
+      <c r="F21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="G21" s="34">
+      <c r="G21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="H21" s="34">
+      <c r="H21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="I21" s="34">
+      <c r="I21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="J21" s="34">
+      <c r="J21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="K21" s="34">
+      <c r="K21" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="L21" s="34">
+      <c r="L21" s="34" t="n">
         <v>72</v>
       </c>
       <c r="M21" s="35"/>
@@ -2891,39 +2974,39 @@
       <c r="BZ21" s="35"/>
       <c r="CA21" s="35"/>
     </row>
-    <row r="22" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="31" t="s">
         <v>57</v>
       </c>
       <c r="B22" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="38"/>
-      <c r="D22" s="34">
+      <c r="C22" s="39"/>
+      <c r="D22" s="34" t="n">
         <v>400</v>
       </c>
       <c r="E22" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="F22" s="34">
+      <c r="F22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="G22" s="34">
+      <c r="G22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="H22" s="34">
+      <c r="H22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="I22" s="34">
+      <c r="I22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="J22" s="34">
+      <c r="J22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="K22" s="34">
+      <c r="K22" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="L22" s="34">
+      <c r="L22" s="34" t="n">
         <v>400</v>
       </c>
       <c r="M22" s="35"/>
@@ -2994,7 +3077,7 @@
       <c r="BZ22" s="35"/>
       <c r="CA22" s="35"/>
     </row>
-    <row r="23" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="31" t="s">
         <v>60</v>
       </c>
@@ -3097,7 +3180,7 @@
       <c r="BZ23" s="35"/>
       <c r="CA23" s="35"/>
     </row>
-    <row r="24" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
         <v>64</v>
       </c>
@@ -3200,39 +3283,39 @@
       <c r="BZ24" s="35"/>
       <c r="CA24" s="35"/>
     </row>
-    <row r="25" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="31" t="s">
         <v>68</v>
       </c>
       <c r="B25" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="38"/>
-      <c r="D25" s="34">
+      <c r="C25" s="39"/>
+      <c r="D25" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="F25" s="34">
+      <c r="F25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="34">
+      <c r="G25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H25" s="34">
+      <c r="H25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I25" s="34">
+      <c r="I25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J25" s="34">
+      <c r="J25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K25" s="34">
+      <c r="K25" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L25" s="34">
+      <c r="L25" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M25" s="35"/>
@@ -3303,39 +3386,39 @@
       <c r="BZ25" s="35"/>
       <c r="CA25" s="35"/>
     </row>
-    <row r="26" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="31" t="s">
         <v>71</v>
       </c>
       <c r="B26" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="38"/>
-      <c r="D26" s="34">
+      <c r="C26" s="39"/>
+      <c r="D26" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="34">
+      <c r="F26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="34">
+      <c r="G26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="34">
+      <c r="H26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I26" s="34">
+      <c r="I26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J26" s="34">
+      <c r="J26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K26" s="34">
+      <c r="K26" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L26" s="34">
+      <c r="L26" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M26" s="35"/>
@@ -3406,7 +3489,7 @@
       <c r="BZ26" s="35"/>
       <c r="CA26" s="35"/>
     </row>
-    <row r="27" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="31" t="s">
         <v>74</v>
       </c>
@@ -3414,31 +3497,31 @@
         <v>75</v>
       </c>
       <c r="C27" s="32"/>
-      <c r="D27" s="34">
+      <c r="D27" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F27" s="34">
+      <c r="F27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="34">
+      <c r="G27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="34">
+      <c r="H27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I27" s="34">
+      <c r="I27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="34">
+      <c r="J27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K27" s="34">
+      <c r="K27" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L27" s="34">
+      <c r="L27" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M27" s="35"/>
@@ -3509,7 +3592,7 @@
       <c r="BZ27" s="35"/>
       <c r="CA27" s="35"/>
     </row>
-    <row r="28" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="31" t="s">
         <v>77</v>
       </c>
@@ -3517,31 +3600,31 @@
         <v>78</v>
       </c>
       <c r="C28" s="32"/>
-      <c r="D28" s="34">
+      <c r="D28" s="34" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="F28" s="34">
+      <c r="F28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="34">
+      <c r="G28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="34">
+      <c r="H28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I28" s="34">
+      <c r="I28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J28" s="34">
+      <c r="J28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K28" s="34">
+      <c r="K28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L28" s="34">
+      <c r="L28" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M28" s="35"/>
@@ -3612,14 +3695,14 @@
       <c r="BZ28" s="35"/>
       <c r="CA28" s="35"/>
     </row>
-    <row r="29" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
         <v>80</v>
       </c>
       <c r="B29" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="38"/>
+      <c r="C29" s="39"/>
       <c r="D29" s="34" t="s">
         <v>82</v>
       </c>
@@ -3715,18 +3798,18 @@
       <c r="BZ29" s="35"/>
       <c r="CA29" s="35"/>
     </row>
-    <row r="30" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="31" t="s">
         <v>83</v>
       </c>
       <c r="B30" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="38"/>
-      <c r="D30" s="34">
+      <c r="C30" s="39"/>
+      <c r="D30" s="34" t="n">
         <v>50</v>
       </c>
-      <c r="E30" s="34">
+      <c r="E30" s="34" t="n">
         <v>55</v>
       </c>
       <c r="F30" s="34" t="s">
@@ -3818,36 +3901,36 @@
       <c r="BZ30" s="35"/>
       <c r="CA30" s="35"/>
     </row>
-    <row r="31" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="31" t="s">
         <v>86</v>
       </c>
       <c r="B31" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="C31" s="38"/>
-      <c r="D31" s="34">
+      <c r="C31" s="39"/>
+      <c r="D31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="F31" s="34">
+      <c r="F31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G31" s="34">
+      <c r="G31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H31" s="34">
+      <c r="H31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I31" s="34">
+      <c r="I31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J31" s="34">
+      <c r="J31" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K31" s="34">
+      <c r="K31" s="34" t="n">
         <v>55</v>
       </c>
       <c r="L31" s="34" t="s">
@@ -3921,7 +4004,7 @@
       <c r="BZ31" s="35"/>
       <c r="CA31" s="35"/>
     </row>
-    <row r="32" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="s">
         <v>89</v>
       </c>
@@ -4024,14 +4107,14 @@
       <c r="BZ32" s="35"/>
       <c r="CA32" s="35"/>
     </row>
-    <row r="33" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="31" t="s">
         <v>91</v>
       </c>
       <c r="B33" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="C33" s="38"/>
+      <c r="C33" s="39"/>
       <c r="D33" s="34" t="s">
         <v>93</v>
       </c>
@@ -4127,33 +4210,33 @@
       <c r="BZ33" s="35"/>
       <c r="CA33" s="35"/>
     </row>
-    <row r="34" spans="1:79" s="41" customFormat="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="39" t="s">
+    <row r="34" s="42" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="B34" s="39" t="s">
+      <c r="B34" s="40" t="s">
         <v>95</v>
       </c>
       <c r="C34" s="15"/>
-      <c r="D34" s="40"/>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="40"/>
-      <c r="I34" s="40"/>
-      <c r="J34" s="40"/>
-      <c r="K34" s="40"/>
-      <c r="L34" s="40"/>
-      <c r="V34" s="42"/>
-      <c r="W34" s="43"/>
-      <c r="AN34" s="42"/>
-      <c r="AO34" s="43"/>
-      <c r="AX34" s="42"/>
-      <c r="AY34" s="43"/>
-      <c r="BQ34" s="42"/>
-      <c r="BR34" s="43"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="41"/>
+      <c r="G34" s="41"/>
+      <c r="H34" s="41"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="41"/>
+      <c r="K34" s="41"/>
+      <c r="L34" s="41"/>
+      <c r="V34" s="43"/>
+      <c r="W34" s="44"/>
+      <c r="AN34" s="43"/>
+      <c r="AO34" s="44"/>
+      <c r="AX34" s="43"/>
+      <c r="AY34" s="44"/>
+      <c r="BQ34" s="43"/>
+      <c r="BR34" s="44"/>
     </row>
-    <row r="35" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="31" t="s">
         <v>96</v>
       </c>
@@ -4188,82 +4271,82 @@
       <c r="L35" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="M35" s="44"/>
-      <c r="N35" s="44"/>
-      <c r="O35" s="44"/>
-      <c r="P35" s="44"/>
-      <c r="Q35" s="44"/>
-      <c r="R35" s="44"/>
-      <c r="S35" s="44"/>
-      <c r="T35" s="44"/>
-      <c r="U35" s="44"/>
-      <c r="V35" s="45"/>
-      <c r="W35" s="46"/>
-      <c r="X35" s="44"/>
-      <c r="Y35" s="44"/>
-      <c r="Z35" s="44"/>
-      <c r="AA35" s="44"/>
-      <c r="AB35" s="44"/>
-      <c r="AC35" s="44"/>
-      <c r="AD35" s="44"/>
-      <c r="AE35" s="44"/>
-      <c r="AF35" s="44"/>
-      <c r="AG35" s="44"/>
-      <c r="AH35" s="44"/>
-      <c r="AI35" s="44"/>
-      <c r="AJ35" s="44"/>
-      <c r="AK35" s="44"/>
-      <c r="AL35" s="44"/>
-      <c r="AM35" s="44"/>
-      <c r="AN35" s="45"/>
-      <c r="AO35" s="46"/>
-      <c r="AP35" s="44"/>
-      <c r="AQ35" s="44"/>
-      <c r="AR35" s="44"/>
-      <c r="AS35" s="44"/>
-      <c r="AT35" s="44"/>
-      <c r="AU35" s="44"/>
-      <c r="AV35" s="44"/>
-      <c r="AW35" s="44"/>
-      <c r="AX35" s="45"/>
-      <c r="AY35" s="46"/>
-      <c r="AZ35" s="44"/>
-      <c r="BA35" s="44"/>
-      <c r="BB35" s="44"/>
-      <c r="BC35" s="44"/>
-      <c r="BD35" s="44"/>
-      <c r="BE35" s="44"/>
-      <c r="BF35" s="44"/>
-      <c r="BG35" s="44"/>
-      <c r="BH35" s="44"/>
-      <c r="BI35" s="44"/>
-      <c r="BJ35" s="44"/>
-      <c r="BK35" s="44"/>
-      <c r="BL35" s="44"/>
-      <c r="BM35" s="44"/>
-      <c r="BN35" s="44"/>
-      <c r="BO35" s="44"/>
-      <c r="BP35" s="44"/>
-      <c r="BQ35" s="45"/>
-      <c r="BR35" s="46"/>
-      <c r="BS35" s="44"/>
-      <c r="BT35" s="44"/>
-      <c r="BU35" s="44"/>
-      <c r="BV35" s="44"/>
-      <c r="BW35" s="44"/>
-      <c r="BX35" s="44"/>
-      <c r="BY35" s="44"/>
-      <c r="BZ35" s="44"/>
-      <c r="CA35" s="44"/>
+      <c r="M35" s="45"/>
+      <c r="N35" s="45"/>
+      <c r="O35" s="45"/>
+      <c r="P35" s="45"/>
+      <c r="Q35" s="45"/>
+      <c r="R35" s="45"/>
+      <c r="S35" s="45"/>
+      <c r="T35" s="45"/>
+      <c r="U35" s="45"/>
+      <c r="V35" s="46"/>
+      <c r="W35" s="47"/>
+      <c r="X35" s="45"/>
+      <c r="Y35" s="45"/>
+      <c r="Z35" s="45"/>
+      <c r="AA35" s="45"/>
+      <c r="AB35" s="45"/>
+      <c r="AC35" s="45"/>
+      <c r="AD35" s="45"/>
+      <c r="AE35" s="45"/>
+      <c r="AF35" s="45"/>
+      <c r="AG35" s="45"/>
+      <c r="AH35" s="45"/>
+      <c r="AI35" s="45"/>
+      <c r="AJ35" s="45"/>
+      <c r="AK35" s="45"/>
+      <c r="AL35" s="45"/>
+      <c r="AM35" s="45"/>
+      <c r="AN35" s="46"/>
+      <c r="AO35" s="47"/>
+      <c r="AP35" s="45"/>
+      <c r="AQ35" s="45"/>
+      <c r="AR35" s="45"/>
+      <c r="AS35" s="45"/>
+      <c r="AT35" s="45"/>
+      <c r="AU35" s="45"/>
+      <c r="AV35" s="45"/>
+      <c r="AW35" s="45"/>
+      <c r="AX35" s="46"/>
+      <c r="AY35" s="47"/>
+      <c r="AZ35" s="45"/>
+      <c r="BA35" s="45"/>
+      <c r="BB35" s="45"/>
+      <c r="BC35" s="45"/>
+      <c r="BD35" s="45"/>
+      <c r="BE35" s="45"/>
+      <c r="BF35" s="45"/>
+      <c r="BG35" s="45"/>
+      <c r="BH35" s="45"/>
+      <c r="BI35" s="45"/>
+      <c r="BJ35" s="45"/>
+      <c r="BK35" s="45"/>
+      <c r="BL35" s="45"/>
+      <c r="BM35" s="45"/>
+      <c r="BN35" s="45"/>
+      <c r="BO35" s="45"/>
+      <c r="BP35" s="45"/>
+      <c r="BQ35" s="46"/>
+      <c r="BR35" s="47"/>
+      <c r="BS35" s="45"/>
+      <c r="BT35" s="45"/>
+      <c r="BU35" s="45"/>
+      <c r="BV35" s="45"/>
+      <c r="BW35" s="45"/>
+      <c r="BX35" s="45"/>
+      <c r="BY35" s="45"/>
+      <c r="BZ35" s="45"/>
+      <c r="CA35" s="45"/>
     </row>
-    <row r="36" spans="1:79" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="47" t="s">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B36" s="47" t="s">
+      <c r="B36" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="C36" s="38"/>
+      <c r="C36" s="39"/>
       <c r="D36" s="33"/>
       <c r="E36" s="33"/>
       <c r="F36" s="33"/>
@@ -4351,14 +4434,14 @@
       <c r="BZ36" s="35"/>
       <c r="CA36" s="35"/>
     </row>
-    <row r="37" spans="1:79" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="47" t="s">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="48" t="s">
         <v>103</v>
       </c>
-      <c r="B37" s="47" t="s">
+      <c r="B37" s="48" t="s">
         <v>104</v>
       </c>
-      <c r="C37" s="38"/>
+      <c r="C37" s="39"/>
       <c r="D37" s="33"/>
       <c r="E37" s="33"/>
       <c r="F37" s="33"/>
@@ -4446,69 +4529,69 @@
       <c r="BZ37" s="35"/>
       <c r="CA37" s="35"/>
     </row>
-    <row r="38" spans="1:79" s="41" customFormat="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="39" t="s">
+    <row r="38" s="42" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="40" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="39" t="s">
+      <c r="B38" s="40" t="s">
         <v>109</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="D38" s="40"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="40"/>
-      <c r="G38" s="40"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="40"/>
-      <c r="J38" s="40"/>
-      <c r="K38" s="40"/>
-      <c r="L38" s="40"/>
-      <c r="V38" s="42"/>
-      <c r="W38" s="43"/>
-      <c r="AN38" s="42"/>
-      <c r="AO38" s="43"/>
-      <c r="AX38" s="42"/>
-      <c r="AY38" s="43"/>
-      <c r="BQ38" s="42"/>
-      <c r="BR38" s="43"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="41"/>
+      <c r="H38" s="41"/>
+      <c r="I38" s="41"/>
+      <c r="J38" s="41"/>
+      <c r="K38" s="41"/>
+      <c r="L38" s="41"/>
+      <c r="V38" s="43"/>
+      <c r="W38" s="44"/>
+      <c r="AN38" s="43"/>
+      <c r="AO38" s="44"/>
+      <c r="AX38" s="43"/>
+      <c r="AY38" s="44"/>
+      <c r="BQ38" s="43"/>
+      <c r="BR38" s="44"/>
     </row>
-    <row r="39" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="31" t="s">
         <v>14</v>
       </c>
       <c r="B39" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="C39" s="38">
+      <c r="C39" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E39" s="33">
+      <c r="E39" s="33" t="n">
         <v>70</v>
       </c>
-      <c r="F39" s="34">
+      <c r="F39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="G39" s="34">
+      <c r="G39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="H39" s="34">
+      <c r="H39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="I39" s="34">
+      <c r="I39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="J39" s="34">
+      <c r="J39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="K39" s="34">
+      <c r="K39" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="L39" s="34">
+      <c r="L39" s="34" t="n">
         <v>70</v>
       </c>
       <c r="M39" s="35"/>
@@ -4579,41 +4662,41 @@
       <c r="BZ39" s="35"/>
       <c r="CA39" s="35"/>
     </row>
-    <row r="40" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="31" t="s">
         <v>16</v>
       </c>
       <c r="B40" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C40" s="38">
+      <c r="C40" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E40" s="33">
+      <c r="E40" s="33" t="n">
         <v>75</v>
       </c>
-      <c r="F40" s="34">
+      <c r="F40" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="G40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="G40" s="34">
+      <c r="H40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="H40" s="34">
+      <c r="I40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="I40" s="34">
+      <c r="J40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="J40" s="34">
+      <c r="K40" s="34" t="n">
         <v>75</v>
       </c>
-      <c r="K40" s="34">
-        <v>75</v>
-      </c>
-      <c r="L40" s="34">
+      <c r="L40" s="34" t="n">
         <v>75</v>
       </c>
       <c r="M40" s="35"/>
@@ -4684,41 +4767,41 @@
       <c r="BZ40" s="35"/>
       <c r="CA40" s="35"/>
     </row>
-    <row r="41" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="31" t="s">
         <v>18</v>
       </c>
       <c r="B41" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="C41" s="38">
+        <v>114</v>
+      </c>
+      <c r="C41" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E41" s="33">
+      <c r="E41" s="33" t="n">
         <v>60</v>
       </c>
-      <c r="F41" s="34">
+      <c r="F41" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="G41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="G41" s="34">
+      <c r="H41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="H41" s="34">
+      <c r="I41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="I41" s="34">
+      <c r="J41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="J41" s="34">
+      <c r="K41" s="34" t="n">
         <v>60</v>
       </c>
-      <c r="K41" s="34">
-        <v>60</v>
-      </c>
-      <c r="L41" s="34">
+      <c r="L41" s="34" t="n">
         <v>60</v>
       </c>
       <c r="M41" s="35"/>
@@ -4789,41 +4872,41 @@
       <c r="BZ41" s="35"/>
       <c r="CA41" s="35"/>
     </row>
-    <row r="42" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="31" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="31" t="s">
-        <v>114</v>
-      </c>
-      <c r="C42" s="38">
+        <v>116</v>
+      </c>
+      <c r="C42" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E42" s="33">
+      <c r="E42" s="33" t="n">
         <v>90</v>
       </c>
-      <c r="F42" s="34">
+      <c r="F42" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="G42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="G42" s="34">
+      <c r="H42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="H42" s="34">
+      <c r="I42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="I42" s="34">
+      <c r="J42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="J42" s="34">
+      <c r="K42" s="34" t="n">
         <v>90</v>
       </c>
-      <c r="K42" s="34">
-        <v>90</v>
-      </c>
-      <c r="L42" s="34">
+      <c r="L42" s="34" t="n">
         <v>90</v>
       </c>
       <c r="M42" s="35"/>
@@ -4894,41 +4977,41 @@
       <c r="BZ42" s="35"/>
       <c r="CA42" s="35"/>
     </row>
-    <row r="43" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="31" t="s">
         <v>22</v>
       </c>
       <c r="B43" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="C43" s="38">
+        <v>117</v>
+      </c>
+      <c r="C43" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E43" s="33">
+      <c r="E43" s="33" t="n">
         <v>1000</v>
       </c>
-      <c r="F43" s="34">
+      <c r="F43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="G43" s="34">
+      <c r="G43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="H43" s="34">
+      <c r="H43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="I43" s="34">
+      <c r="I43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="J43" s="34">
+      <c r="J43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="K43" s="34">
+      <c r="K43" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="L43" s="34">
+      <c r="L43" s="34" t="n">
         <v>1000</v>
       </c>
       <c r="M43" s="35"/>
@@ -4999,41 +5082,41 @@
       <c r="BZ43" s="35"/>
       <c r="CA43" s="35"/>
     </row>
-    <row r="44" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="31" t="s">
         <v>25</v>
       </c>
       <c r="B44" s="31" t="s">
-        <v>116</v>
-      </c>
-      <c r="C44" s="38">
+        <v>118</v>
+      </c>
+      <c r="C44" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E44" s="33">
+      <c r="E44" s="33" t="n">
         <v>75</v>
       </c>
-      <c r="F44" s="34">
+      <c r="F44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="G44" s="34">
+      <c r="G44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="H44" s="34">
+      <c r="H44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="I44" s="34">
+      <c r="I44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="J44" s="34">
+      <c r="J44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="K44" s="34">
+      <c r="K44" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="L44" s="34">
+      <c r="L44" s="34" t="n">
         <v>500</v>
       </c>
       <c r="M44" s="35"/>
@@ -5104,41 +5187,41 @@
       <c r="BZ44" s="35"/>
       <c r="CA44" s="35"/>
     </row>
-    <row r="45" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="31" t="s">
         <v>29</v>
       </c>
       <c r="B45" s="31" t="s">
-        <v>117</v>
-      </c>
-      <c r="C45" s="38">
+        <v>119</v>
+      </c>
+      <c r="C45" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E45" s="35">
+      <c r="E45" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="F45" s="34">
+      <c r="F45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="G45" s="34">
+      <c r="G45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="H45" s="34">
+      <c r="H45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="I45" s="34">
+      <c r="I45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="J45" s="34">
+      <c r="J45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="K45" s="34">
+      <c r="K45" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="L45" s="34">
+      <c r="L45" s="34" t="n">
         <v>100</v>
       </c>
       <c r="M45" s="35"/>
@@ -5209,41 +5292,41 @@
       <c r="BZ45" s="35"/>
       <c r="CA45" s="35"/>
     </row>
-    <row r="46" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="31" t="s">
         <v>32</v>
       </c>
       <c r="B46" s="31" t="s">
-        <v>118</v>
-      </c>
-      <c r="C46" s="38">
+        <v>120</v>
+      </c>
+      <c r="C46" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E46" s="33">
+      <c r="E46" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F46" s="34">
+      <c r="F46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="G46" s="34">
+      <c r="G46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="H46" s="34">
+      <c r="H46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="I46" s="34">
+      <c r="I46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="J46" s="34">
+      <c r="J46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="K46" s="34">
+      <c r="K46" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="L46" s="34">
+      <c r="L46" s="34" t="n">
         <v>200</v>
       </c>
       <c r="M46" s="35"/>
@@ -5314,41 +5397,41 @@
       <c r="BZ46" s="35"/>
       <c r="CA46" s="35"/>
     </row>
-    <row r="47" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="31" t="s">
         <v>35</v>
       </c>
       <c r="B47" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="C47" s="38">
+        <v>121</v>
+      </c>
+      <c r="C47" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E47" s="33">
+      <c r="E47" s="33" t="n">
         <v>65</v>
       </c>
-      <c r="F47" s="34">
+      <c r="F47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="G47" s="34">
+      <c r="G47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="H47" s="34">
+      <c r="H47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="I47" s="34">
+      <c r="I47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="J47" s="34">
+      <c r="J47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="K47" s="34">
+      <c r="K47" s="34" t="n">
         <v>120</v>
       </c>
-      <c r="L47" s="34">
+      <c r="L47" s="34" t="n">
         <v>120</v>
       </c>
       <c r="M47" s="35"/>
@@ -5419,41 +5502,41 @@
       <c r="BZ47" s="35"/>
       <c r="CA47" s="35"/>
     </row>
-    <row r="48" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="31" t="s">
         <v>39</v>
       </c>
       <c r="B48" s="31" t="s">
-        <v>120</v>
-      </c>
-      <c r="C48" s="38">
+        <v>122</v>
+      </c>
+      <c r="C48" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E48" s="33">
+      <c r="E48" s="33" t="n">
         <v>68</v>
       </c>
-      <c r="F48" s="34">
+      <c r="F48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="G48" s="34">
+      <c r="G48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="H48" s="34">
+      <c r="H48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="I48" s="34">
+      <c r="I48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="J48" s="34">
+      <c r="J48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="K48" s="34">
+      <c r="K48" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="L48" s="34">
+      <c r="L48" s="34" t="n">
         <v>20</v>
       </c>
       <c r="M48" s="35"/>
@@ -5524,41 +5607,41 @@
       <c r="BZ48" s="35"/>
       <c r="CA48" s="35"/>
     </row>
-    <row r="49" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="31" t="s">
         <v>43</v>
       </c>
       <c r="B49" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="C49" s="38">
+      <c r="C49" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E49" s="33">
+      <c r="E49" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F49" s="34">
+      <c r="F49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="G49" s="34">
+      <c r="G49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="H49" s="34">
+      <c r="H49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="I49" s="34">
+      <c r="I49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="J49" s="34">
+      <c r="J49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="K49" s="34">
+      <c r="K49" s="34" t="n">
         <v>70</v>
       </c>
-      <c r="L49" s="34">
+      <c r="L49" s="34" t="n">
         <v>70</v>
       </c>
       <c r="M49" s="35"/>
@@ -5629,41 +5712,41 @@
       <c r="BZ49" s="35"/>
       <c r="CA49" s="35"/>
     </row>
-    <row r="50" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="31" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="C50" s="38">
+        <v>123</v>
+      </c>
+      <c r="C50" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E50" s="33">
+      <c r="E50" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F50" s="34">
+      <c r="F50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="G50" s="34">
+      <c r="G50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="H50" s="34">
+      <c r="H50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="I50" s="34">
+      <c r="I50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="J50" s="34">
+      <c r="J50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="K50" s="34">
+      <c r="K50" s="34" t="n">
         <v>150</v>
       </c>
-      <c r="L50" s="34">
+      <c r="L50" s="34" t="n">
         <v>150</v>
       </c>
       <c r="M50" s="35"/>
@@ -5734,41 +5817,41 @@
       <c r="BZ50" s="35"/>
       <c r="CA50" s="35"/>
     </row>
-    <row r="51" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="31" t="s">
         <v>51</v>
       </c>
       <c r="B51" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="C51" s="38">
+        <v>124</v>
+      </c>
+      <c r="C51" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="33" t="s">
         <v>111</v>
       </c>
       <c r="E51" s="33" t="s">
-        <v>123</v>
-      </c>
-      <c r="F51" s="34">
+        <v>125</v>
+      </c>
+      <c r="F51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G51" s="34">
+      <c r="G51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H51" s="34">
+      <c r="H51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I51" s="34">
+      <c r="I51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J51" s="34">
+      <c r="J51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K51" s="34">
+      <c r="K51" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="L51" s="34">
+      <c r="L51" s="34" t="n">
         <v>55</v>
       </c>
       <c r="M51" s="35"/>
@@ -5839,41 +5922,41 @@
       <c r="BZ51" s="35"/>
       <c r="CA51" s="35"/>
     </row>
-    <row r="52" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="31" t="s">
         <v>54</v>
       </c>
       <c r="B52" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="C52" s="38">
+        <v>126</v>
+      </c>
+      <c r="C52" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="33" t="s">
         <v>111</v>
       </c>
       <c r="E52" s="33" t="s">
-        <v>123</v>
-      </c>
-      <c r="F52" s="34">
+        <v>125</v>
+      </c>
+      <c r="F52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="G52" s="34">
+      <c r="G52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="H52" s="34">
+      <c r="H52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="I52" s="34">
+      <c r="I52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="J52" s="34">
+      <c r="J52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="K52" s="34">
+      <c r="K52" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="L52" s="34">
+      <c r="L52" s="34" t="n">
         <v>72</v>
       </c>
       <c r="M52" s="35"/>
@@ -5944,41 +6027,41 @@
       <c r="BZ52" s="35"/>
       <c r="CA52" s="35"/>
     </row>
-    <row r="53" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="31" t="s">
         <v>57</v>
       </c>
       <c r="B53" s="31" t="s">
-        <v>125</v>
-      </c>
-      <c r="C53" s="38">
+        <v>127</v>
+      </c>
+      <c r="C53" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D53" s="33" t="s">
         <v>111</v>
       </c>
       <c r="E53" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F53" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="G53" s="34">
+        <v>129</v>
+      </c>
+      <c r="G53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="H53" s="34">
+      <c r="H53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="I53" s="34">
+      <c r="I53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="J53" s="34">
+      <c r="J53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="K53" s="34">
+      <c r="K53" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="L53" s="34">
+      <c r="L53" s="34" t="n">
         <v>400</v>
       </c>
       <c r="M53" s="35"/>
@@ -6049,21 +6132,21 @@
       <c r="BZ53" s="35"/>
       <c r="CA53" s="35"/>
     </row>
-    <row r="54" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="31" t="s">
         <v>60</v>
       </c>
       <c r="B54" s="31" t="s">
-        <v>127</v>
-      </c>
-      <c r="C54" s="38">
+        <v>130</v>
+      </c>
+      <c r="C54" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D54" s="33" t="s">
         <v>111</v>
       </c>
       <c r="E54" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F54" s="34" t="s">
         <v>62</v>
@@ -6154,20 +6237,20 @@
       <c r="BZ54" s="35"/>
       <c r="CA54" s="35"/>
     </row>
-    <row r="55" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="31" t="s">
         <v>64</v>
       </c>
       <c r="B55" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="C55" s="38">
+        <v>131</v>
+      </c>
+      <c r="C55" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E55" s="33">
+      <c r="E55" s="33" t="n">
         <v>72</v>
       </c>
       <c r="F55" s="34" t="s">
@@ -6259,41 +6342,41 @@
       <c r="BZ55" s="35"/>
       <c r="CA55" s="35"/>
     </row>
-    <row r="56" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="31" t="s">
         <v>68</v>
       </c>
       <c r="B56" s="31" t="s">
-        <v>129</v>
-      </c>
-      <c r="C56" s="38">
+        <v>132</v>
+      </c>
+      <c r="C56" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E56" s="33">
+      <c r="E56" s="33" t="n">
         <v>720</v>
       </c>
-      <c r="F56" s="34">
+      <c r="F56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G56" s="34">
+      <c r="G56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H56" s="34">
+      <c r="H56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I56" s="34">
+      <c r="I56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J56" s="34">
+      <c r="J56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K56" s="34">
+      <c r="K56" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L56" s="34">
+      <c r="L56" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M56" s="35"/>
@@ -6364,41 +6447,41 @@
       <c r="BZ56" s="35"/>
       <c r="CA56" s="35"/>
     </row>
-    <row r="57" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="31" t="s">
         <v>71</v>
       </c>
       <c r="B57" s="31" t="s">
-        <v>130</v>
-      </c>
-      <c r="C57" s="32">
+        <v>133</v>
+      </c>
+      <c r="C57" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E57" s="33">
+      <c r="E57" s="33" t="n">
         <v>48</v>
       </c>
-      <c r="F57" s="34">
+      <c r="F57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G57" s="34">
+      <c r="G57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H57" s="34">
+      <c r="H57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I57" s="34">
+      <c r="I57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J57" s="34">
+      <c r="J57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K57" s="34">
+      <c r="K57" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L57" s="34">
+      <c r="L57" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M57" s="35"/>
@@ -6469,41 +6552,41 @@
       <c r="BZ57" s="35"/>
       <c r="CA57" s="35"/>
     </row>
-    <row r="58" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="31" t="s">
         <v>74</v>
       </c>
       <c r="B58" s="31" t="s">
-        <v>131</v>
-      </c>
-      <c r="C58" s="32">
+        <v>134</v>
+      </c>
+      <c r="C58" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D58" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E58" s="33">
+      <c r="E58" s="33" t="n">
         <v>72</v>
       </c>
-      <c r="F58" s="34">
+      <c r="F58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="34">
+      <c r="G58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H58" s="34">
+      <c r="H58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I58" s="34">
+      <c r="I58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J58" s="34">
+      <c r="J58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K58" s="34">
+      <c r="K58" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L58" s="34">
+      <c r="L58" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M58" s="35"/>
@@ -6574,41 +6657,41 @@
       <c r="BZ58" s="35"/>
       <c r="CA58" s="35"/>
     </row>
-    <row r="59" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="31" t="s">
         <v>77</v>
       </c>
       <c r="B59" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="C59" s="38">
+        <v>135</v>
+      </c>
+      <c r="C59" s="39" t="n">
         <v>0</v>
       </c>
       <c r="D59" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="E59" s="33">
+      <c r="E59" s="33" t="n">
         <v>84</v>
       </c>
-      <c r="F59" s="34">
+      <c r="F59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="G59" s="34">
+      <c r="G59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="H59" s="34">
+      <c r="H59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I59" s="34">
+      <c r="I59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="J59" s="34">
+      <c r="J59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K59" s="34">
+      <c r="K59" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="L59" s="34">
+      <c r="L59" s="34" t="n">
         <v>1</v>
       </c>
       <c r="M59" s="35"/>
@@ -6679,41 +6762,41 @@
       <c r="BZ59" s="35"/>
       <c r="CA59" s="35"/>
     </row>
-    <row r="60" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="31" t="s">
         <v>83</v>
       </c>
       <c r="B60" s="31" t="s">
-        <v>133</v>
-      </c>
-      <c r="C60" s="32">
+        <v>136</v>
+      </c>
+      <c r="C60" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D60" s="33" t="s">
         <v>111</v>
       </c>
       <c r="E60" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="F60" s="34">
+        <v>137</v>
+      </c>
+      <c r="F60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G60" s="34">
+      <c r="G60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H60" s="34">
+      <c r="H60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I60" s="34">
+      <c r="I60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J60" s="34">
+      <c r="J60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K60" s="34">
+      <c r="K60" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="L60" s="34">
+      <c r="L60" s="34" t="n">
         <v>55</v>
       </c>
       <c r="M60" s="35"/>
@@ -6784,38 +6867,38 @@
       <c r="BZ60" s="35"/>
       <c r="CA60" s="35"/>
     </row>
-    <row r="61" spans="1:79" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="31" t="s">
         <v>86</v>
       </c>
       <c r="B61" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="C61" s="32">
+        <v>138</v>
+      </c>
+      <c r="C61" s="32" t="n">
         <v>0.05</v>
       </c>
       <c r="D61" s="33" t="s">
         <v>111</v>
       </c>
       <c r="E61" s="33" t="s">
-        <v>136</v>
-      </c>
-      <c r="F61" s="34">
+        <v>139</v>
+      </c>
+      <c r="F61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="G61" s="34">
+      <c r="G61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="H61" s="34">
+      <c r="H61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="I61" s="34">
+      <c r="I61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="J61" s="34">
+      <c r="J61" s="34" t="n">
         <v>55</v>
       </c>
-      <c r="K61" s="34">
+      <c r="K61" s="34" t="n">
         <v>55</v>
       </c>
       <c r="L61" s="34" t="s">
@@ -6891,12 +6974,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="M8:ZZ33 M39:ZZ61">
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>#REF!&lt;&gt;M8</formula>
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>#ref!&lt;&gt;M8</formula>
     </cfRule>
   </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>